<commit_message>
Sync derived formats with corrected source; codify LaTeX-first workflow
- EPUB rebuilt from source: all ~45 recent corrections verified present
  (index conventions, simplex caption, Dijkstra direction, etc.);
  33/33 xhtml parse clean; 202 images all carry alt text; 162 figure +
  64 table captions (two duplicate ch2 figures removed)
- html/ regenerated from the new EPUB (32 chapters, clean XHTML)
- Figures-and-AltText spreadsheet regenerated: 162 rows, 0 empty alt
- NEW CORRECTIONS-WORKFLOW.md: LaTeX is the single source of truth;
  fix source first, then rebuild PDF -> EPUB -> HTML and commit built
  artifacts together; scripts/rebuild-derived.sh runs the derived steps
- epub-build/WORKFLOW.md: rebuild gotchas appended (stale snippet PNGs,
  spreadsheet args, dvipng/tidy absence, dijkstra macro placeholder)

PDF rebuild (pdflatexmk, author machine) is the remaining step before
the reviewer copy goes out.
</commit_message>
<xml_diff>
--- a/Intro-Math-Programming/baseText/book/Figures-and-AltText-book1-filled.xlsx
+++ b/Intro-Math-Programming/baseText/book/Figures-and-AltText-book1-filled.xlsx
@@ -392,7 +392,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y165"/>
+  <dimension ref="A1:Y163"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="10" customWidth="1" style="14" min="1" max="1"/>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>Cone-shaped feasible region on x1-x2 axes: blue shading between the lines s1 = 0 (red, lower...</t>
+          <t>Cone-shaped feasible region between the lines s1 = 0 and s3 = 0, with s2 = 0 above, shaded blue and marked...</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>Cone-shaped feasible region on x1-x2 axes: blue shading between the lines s1 = 0 (red, lower boundary) and s3 = 0 (orange, upper boundary), with the line s2 = 0 (teal) crossing above; red square markers sit at (0,0), (0,1), and (2,3).</t>
+          <t>The same cone-shaped region between s1 = 0 and s3 = 0 with s2 = 0 above, shaded blue and marked with red squares at (0,0), (0,1), and (2,3), used to discuss which basic solutions are feasible.</t>
         </is>
       </c>
       <c r="D38" s="17" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>The same cone-shaped region between s1 = 0 and s3 = 0 with s2 = 0 above, shaded blue and marked...</t>
+          <t>Recession cone plot: shaded blue cone between the lines s1 = 0 (red) and s3 = 0 (orange) with s2 =...</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>The same cone-shaped region between s1 = 0 and s3 = 0 with s2 = 0 above, shaded blue and marked with red squares at (0,0), (0,1), and (2,3), used to discuss which basic solutions are feasible.</t>
+          <t>The same recession cone between s1 = 0 and s3 = 0 with the line x1 + x2 = 1 crossing it, used to identify the extreme rays of the cone.</t>
         </is>
       </c>
       <c r="D39" s="17" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>Recession cone plot: shaded blue cone between the lines s1 = 0 (red) and s3 = 0 (orange) with s2 =...</t>
+          <t>Zoomed view of the normalization segment: the line x1 + x2 = 1 crosses the shaded cone between s1 =...</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>The same recession cone between s1 = 0 and s3 = 0 with the line x1 + x2 = 1 crossing it, used to identify the extreme rays of the cone.</t>
+          <t>Recession cone plot: shaded blue cone between the lines s1 = 0 (red) and s3 = 0 (orange) with s2 = 0 (teal) above; the normalization line x1 + x2 = 1 is drawn crossing the cone near the origin.</t>
         </is>
       </c>
       <c r="D40" s="17" t="inlineStr">
@@ -1486,17 +1486,17 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>The same recession cone between s1 = 0 and s3 = 0 with the line x1 + x2 = 1 crossing it, used to...</t>
+          <t>A convex combination of the points x and y is given by z = λx + (1 − λ)y with any λ ∈ [0,1]. Here we demonstrate this using λ = 2∕3.</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>The same recession cone between s1 = 0 and s3 = 0 with the line x1 + x2 = 1 crossing it, used to identify the extreme rays of the cone.</t>
+          <t>Schematic of a convex combination on a 2D plane: two black points x and y are joined by a line segment, with a red point z placed one-third of the way from y to x to illustrate z = lambda*x + (1-lambda)*y for lambda = 2/3.</t>
         </is>
       </c>
       <c r="D41" s="17" t="inlineStr">
@@ -1512,17 +1512,18 @@
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>5.13</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>Zoomed view of the normalization segment: the line x1 + x2 = 1 crosses the shaded cone between s1 =...</t>
+          <t>A convex set and a non-convex set.</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>Zoomed view of the normalization segment: the line x1 + x2 = 1 crosses the shaded cone between s1 = 0 and s3 = 0, and two red square points mark where the extreme rays meet the line.</t>
+          <t>PIC
+Two side-by-side shapes contrasting a convex set (a tilted gray ellipse) with a non-convex set (a curvy gray blob with a notch); a chord between two interior dots leaves the second shape, demonstrating non-convexity.</t>
         </is>
       </c>
       <c r="D42" s="17" t="inlineStr">
@@ -1538,17 +1539,21 @@
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>A convex combination of the points x and y is given by z = λx + (1 − λ)y with any λ ∈ [0,1]. Here we demonstrate this using λ = 2∕3.</t>
+          <t>Examples of convex sets: a hyperplane, a halfspace, a polyhedron, a ball, and a second-order cone.</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>Schematic of a convex combination on a 2D plane: two black points x and y are joined by a line segment, with a red point z placed one-third of the way from y to x to illustrate z = lambda*x + (1-lambda)*y for lambda = 2/3.</t>
+          <t>PIC
+PIC
+A green shaded polyhedron (a tilted quadrilateral) in the x1-x2 plane, labeled Polyhedron.
+A shaded ball (disk) in the x1-x2 plane, an example of a convex set.
+An orange shaded triangle opening upward from the origin in the x1-x2 plane, labeled the Second Order Cone: the set of (x, t) with norm of x squared at most t squared.</t>
         </is>
       </c>
       <c r="D43" s="17" t="inlineStr">
@@ -1564,18 +1569,17 @@
     <row r="44">
       <c r="A44" s="16" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>A convex set and a non-convex set.</t>
+          <t>The green intersection of the convex sets that are the ball and the polytope is also convex. This can be seen by considering any points x,y ∈Ball ∩Polytope. Since Ball is convex, the line segment between x and y is completely contained in Ball. And similarly, the line segment is completely contained in Polytope. Hence, the line segment is also contained in the intersection. This is how we can reason that the intersection is also convex.</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>A convex set: an ellipse-shaped region.
-Two side-by-side shapes contrasting a convex set (a tilted gray ellipse) with a non-convex set (a curvy gray blob with a notch); a chord between two interior dots leaves the second shape, demonstrating non-convexity.</t>
+          <t>The green intersection of the ball and the polytope, which is again a convex set.</t>
         </is>
       </c>
       <c r="D44" s="17" t="inlineStr">
@@ -1591,21 +1595,17 @@
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>Examples of convex sets: a hyperplane, a halfspace, a polyhedron, a ball, and a second-order cone.</t>
+          <t>A number line showing that the objective value at z lies between the objective values at x and y.</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>A hyperplane in the plane: the line through the origin.
-A halfspace: all points on one side of a line.
-A green shaded polyhedron (a tilted quadrilateral) in the x1-x2 plane, labeled Polyhedron.
-A shaded ball (disk) in the x1-x2 plane, an example of a convex set.
-An orange shaded triangle opening upward from the origin in the x1-x2 plane, labeled the Second Order Cone: the set of (x, t) with norm of x squared at most t squared.</t>
+          <t>One-dimensional number line showing c^T z between c^T x and c^T y. Three dots mark min and max of {c^T x, c^T y} and the convex combination c^T z = lambda c^T x + (1-lambda) c^T y in between.</t>
         </is>
       </c>
       <c r="D45" s="17" t="inlineStr">
@@ -1621,17 +1621,17 @@
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>The green intersection of the convex sets that are the ball and the polytope is also convex. This can be seen by considering any points x,y ∈Ball ∩Polytope. Since Ball is convex, the line segment between x and y is completely contained in Ball. And similarly, the line segment is completely contained in Polytope. Hence, the line segment is also contained in the intersection. This is how we can reason that the intersection is also convex.</t>
+          <t>Two-dimensional plot of a quadrilateral polytope with vertices (0,0), (1,2), (3,2), (4,0).</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>The green intersection of the ball and the polytope, which is again a convex set.</t>
+          <t>Two-dimensional plot of a quadrilateral polytope with vertices (0,0), (1,2), (3,2), (4,0). A green vertex v and two interior red points x and y each show short arrows v +/- epsilon*d, distinguishing perturbations that stay inside from those that leave the polytope.</t>
         </is>
       </c>
       <c r="D46" s="17" t="inlineStr">
@@ -1647,17 +1647,17 @@
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>A number line showing that the objective value at z lies between the objective values at x and y.</t>
+          <t>Feasible region with the lines s1 = 0, s2 = 0, s3 = 0 marking where each slack variable vanishes; the extreme points (0,0), (0,1), and (2,3) are marked.</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>One-dimensional number line showing c^T z between c^T x and c^T y. Three dots mark min and max of {c^T x, c^T y} and the convex combination c^T z = lambda c^T x + (1-lambda) c^T y in between.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D47" s="17" t="inlineStr">
@@ -1673,17 +1673,17 @@
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of a quadrilateral polytope with vertices (0,0), (1,2), (3,2), (4,0).</t>
+          <t>Correspondence between original and canonical form solutions.</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of a quadrilateral polytope with vertices (0,0), (1,2), (3,2), (4,0). A green vertex v and two interior red points x and y each show short arrows v +/- epsilon*d, distinguishing perturbations that stay inside from those that leave the polytope.</t>
+          <t>Two-row diagram: Original LP (min or max, unrestricted variables, inequalities) connected by arrows labeled 'variable transformations / interpret in original space' to Transformed LP in Canonical Form (max, all equalities, variables &gt;= 0); below, Solution to Original LP is connected to Solution to Transformed LP by 'encode to canonical form / map back (e.g., x_j = x_j-plus minus x_j-minus)'.</t>
         </is>
       </c>
       <c r="D48" s="17" t="inlineStr">
@@ -1699,17 +1699,17 @@
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>Feasible region with the lines s1=0, s2=0, s3=0 marking where each slack variable vanishes; basic...</t>
+          <t>When can you use canonical form?</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>Feasible region with the lines s1=0, s2=0, s3=0 marking where each slack variable vanishes; basic solutions are marked with red squares.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
@@ -1725,43 +1725,55 @@
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>Correspondence between original and canonical form solutions.</t>
+          <t>If an optimal point exists, it is one of the vertices of the polyhedron. The simplex algorithm searches for optimal points by moving between adjacent vertices in a direction that increases the value of the objective function until it finds an optimal vertex.</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>Two-row diagram: Original LP (min or max, unrestricted variables, inequalities) connected by arrows labeled 'variable transformations / interpret in original space' to Transformed LP in Canonical Form (max, all equalities, variables &gt;= 0); below, Solution to Original LP is connected to Solution to Transformed LP by 'encode to canonical form / map back (e.g., x_j = x_j-plus minus x_j-minus)'.</t>
+          <t>PIC
+PIC</t>
         </is>
       </c>
       <c r="D50" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E50" s="17" t="inlineStr"/>
-      <c r="F50" s="17" t="inlineStr"/>
+          <t>CC BY 3.0 US</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>Foundations of Applied Mathematics (BYU ACME), Volume 2, Simplex lab</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>Foundations of Applied Mathematics, BYU ACME labs, CC BY 3.0 US, https://github.com/Foundations-of-Applied-Mathematics</t>
+        </is>
+      </c>
       <c r="G50" s="17" t="inlineStr"/>
       <c r="H50" s="17" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>When can you use canonical form?</t>
+          <t>The same linear program seen from every vertex: each basic feasible solution has its own dictionary, whose objective row reveals whether a better neighbor exists. The orange arrows trace the pivots taken in the text, (0,0) → (0,7) → (4,5); at (4,5) all objective coefficients are negative, certifying optimality.</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>When can you use canonical form? Flowchart from the original LP through slack variables (obvious BFS) or artificial variables (Phase I).</t>
+          <t>Blue feasible region with constraint lines x+y=9 (red), 2x+y=16 (teal), and x+2y=... (orange); the optimum is marked with a red dot at (4,5) and vertices (0,0), (0,7), (7,2), (8,0) are labeled.
+PIC
+PIC
+PIC</t>
         </is>
       </c>
       <c r="D51" s="17" t="inlineStr">
@@ -1777,55 +1789,43 @@
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>If an optimal point exists, it is one of the vertices of the polyhedron. The simplex algorithm searches for optimal points by moving between adjacent vertices in a direction that increases the value of the objective function until it finds an optimal vertex.</t>
+          <t>The feasible region with the basis and objective value at every vertex; two possible simplex paths (solid and dashed) both lead to the optimal vertex (4,5).</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>PIC
-A polytope with a path of improving edges leading to the optimal vertex x*.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D52" s="17" t="inlineStr">
         <is>
-          <t>CC BY 3.0 US</t>
-        </is>
-      </c>
-      <c r="E52" s="17" t="inlineStr">
-        <is>
-          <t>Foundations of Applied Mathematics (BYU ACME), Volume 2, Simplex lab</t>
-        </is>
-      </c>
-      <c r="F52" s="17" t="inlineStr">
-        <is>
-          <t>Foundations of Applied Mathematics, BYU ACME labs, CC BY 3.0 US, https://github.com/Foundations-of-Applied-Mathematics</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr"/>
+      <c r="F52" s="17" t="inlineStr"/>
       <c r="G52" s="17" t="inlineStr"/>
       <c r="H52" s="17" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>The same linear program seen from every vertex: each basic feasible solution has its own dictionary, whose objective row reveals whether a better neighbor exists. The orange arrows trace the pivots taken in the text, (0,0) → (0,7) → (4,5); at (4,5) all objective coefficients are negative, certifying optimality.</t>
+          <t>Feasible region after adding the constraint 2x+y&gt;=5: the pink triangle near the origin becomes infeasible.</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>Blue feasible region with constraint lines x+y=9 (red), 2x+y=16 (teal), and x+2y=... (orange); the optimum is marked with a red dot at (4,5) and vertices (0,0), (0,7), (7,2), (8,0) are labeled.
-PIC
-PIC
-PIC</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D53" s="17" t="inlineStr">
@@ -1841,17 +1841,21 @@
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.7</t>
         </is>
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>The feasible region with the basis and objective value at every vertex; the simplex path leads to...</t>
+          <t>The feasible region defined by x1 − x2 ≤ 1, 2x1 − x2 ≤ 3, x1,x2 ≥ 0: an unbounded region extending to the upper right.</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>The feasible region with the basis and objective value at every vertex; the simplex path leads to the optimum (4,5) with z=23.</t>
+          <t>PIC
+PIC
+PIC
+PIC
+Desmos plot of the feasible region defined by x1-x2&lt;=1, 2x1-x2&lt;=3, x1,x2&gt;=0: an unbounded region extending to the right in the first quadrant, illustrating the unbounded LP example.</t>
         </is>
       </c>
       <c r="D54" s="17" t="inlineStr">
@@ -1867,17 +1871,17 @@
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>Feasible region after adding the constraint 2x+y&gt;=5: the pink triangle near the origin becomes infeasible.</t>
+          <t>The feasible region with vertices labeled A, B, C, D, used to identify basic and nonbasic variables and to trace pivots between adjacent basic feasible solutions.</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>Feasible region after adding the constraint 2x+y&gt;=5: the pink triangle near the origin becomes infeasible.</t>
+          <t>Desmos graph of a 2-variable LP feasible region with vertices labeled A, B, C, D used to identify basic and nonbasic variables and to trace pivot moves between adjacent basic feasible solutions.</t>
         </is>
       </c>
       <c r="D55" s="17" t="inlineStr">
@@ -1893,17 +1897,17 @@
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>7.7</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>Desmos plot of the feasible region defined by x1-x2&lt;=1, 2x1-x2&lt;=3, x1,x2&gt;=0: an unbounded region...</t>
+          <t>The three bases of this subsection, seen geometrically. Each basis fixes the nonbasic variables at zero, which places the basic solution at the intersection of two constraint boundaries. Bases {x1,x2} and {s1,s2} give basic feasible solutions at the vertices (6,5) and (0,0) (filled dots). Basis {x1,s2} gives the basic solution (16,0) (open dot), the intersection of the x1-axis ( x2 = 0) with the boundary x1 + 2x2 = 16 ( s1 = 0); it violates 5x1 + 3x2 ≤ 45, so it is an infeasible basic solution and lies outside the region.</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>Desmos plot of the feasible region defined by x1-x2&lt;=1, 2x1-x2&lt;=3, x1,x2&gt;=0: an unbounded region extending to the right in the first quadrant, illustrating the unbounded LP example.</t>
+          <t>Feasible region shaded blue for x1+2x2&lt;=16 (orange line) and 5x1+3x2&lt;=45 (teal line) with corner points (0,0), (0,8), (6,5), and (9,0) marked as filled dots; labels give the basis at several points, for example B={x1,x2} at (6,5), and the point (16,0) is drawn as an open circle labeled an infeasible basic solution.</t>
         </is>
       </c>
       <c r="D56" s="17" t="inlineStr">
@@ -1919,17 +1923,18 @@
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>7.8</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B57" s="17" t="inlineStr">
         <is>
-          <t>Desmos graph of a 2-variable LP feasible region with vertices labeled A, B, C, D used to identify...</t>
+          <t>Feasible region with level curves of the objective z = cxx + 3y for several slopes: for cx ∈ [1.5,3] the optimal vertex (and basis) does not change.</t>
         </is>
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>Desmos graph of a 2-variable LP feasible region with vertices labeled A, B, C, D used to identify basic and nonbasic variables and to trace pivot moves between adjacent basic feasible solutions.</t>
+          <t>Feasible region shaded blue with vertices (0,0), (0,7), (4,5), (7,2), (8,0); parallel red level lines x+y=7, x+y=9, and x+y=10 sweep across the region, with a green line 2x+y=16 and a brown line showing a modified constraint.
+Sensitivity analysis visualization showing how the optimal solution changes as objective function coefficients vary.</t>
         </is>
       </c>
       <c r="D57" s="17" t="inlineStr">
@@ -1945,17 +1950,17 @@
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>The three bases of this subsection, seen geometrically. Each basis fixes the nonbasic variables at zero, which places the basic solution at the intersection of two constraint boundaries. Bases {x1,x2} and {s1,s2} give basic feasible solutions at the vertices (6,5) and (0,0) (filled dots). Basis {x1,s2} gives the basic solution (16,0) (open dot), the intersection of the x1-axis ( x2 = 0) with the boundary x1 + 2x2 = 16 ( s1 = 0); it violates 5x1 + 3x2 ≤ 45, so it is an infeasible basic solution and lies outside the region.</t>
+          <t>Excel’s Solver Results dialog with the option to generate a Sensitivity report selected.</t>
         </is>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>Feasible region shaded blue for x1+2x2&lt;=16 (orange line) and 5x1+3x2&lt;=45 (teal line) with corner points (0,0), (0,8), (6,5), and (9,0) marked as filled dots; labels give the basis at several points, for example B={x1,x2} at (6,5), and the point (16,0) is drawn as an open circle labeled an infeasible basic solution.</t>
+          <t>A Microsoft Excel Solver Results dialog box showing a successful optimization, with options to keep the solution or restore original values, and report type selections.</t>
         </is>
       </c>
       <c r="D58" s="17" t="inlineStr">
@@ -1971,18 +1976,17 @@
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B59" s="17" t="inlineStr">
         <is>
-          <t>Feasible region in the x-y plane with several level curves of the objective z = c_x x + 3y drawn...</t>
+          <t>An Excel worksheet laid out for Solver, with decision-variable cells, a SUMPRODUCT objective, and constraint formulas.</t>
         </is>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>Feasible region shaded blue with vertices (0,0), (0,7), (4,5), (7,2), (8,0); parallel red level lines x+y=7, x+y=9, and x+y=10 sweep across the region, with a green line 2x+y=16 and a brown line showing a modified constraint.
-Sensitivity analysis visualization showing how the optimal solution changes as objective function coefficients vary.</t>
+          <t>An Excel spreadsheet setup for a linear programming problem with decision variables in yellow cells. Constraints are defined with coefficients, totals, and right-hand side values.</t>
         </is>
       </c>
       <c r="D59" s="17" t="inlineStr">
@@ -1998,17 +2002,17 @@
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>Screenshot of Excel’s Solver Results dialog with the option to generate a Sensitivity report...</t>
+          <t>The Solver sensitivity report: variable cells (final value, reduced cost, objective coefficient, allowable increase/decrease) and constraints (final value, shadow price, RHS, allowable increase/decrease).</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>A Microsoft Excel Solver Results dialog box showing a successful optimization, with options to keep the solution or restore original values, and report type selections.</t>
+          <t>A Microsoft Excel Solver sensitivity analysis report showing Variable Cells and Constraints sections with columns for Final Value, Reduced Cost, and Shadow Price.</t>
         </is>
       </c>
       <c r="D60" s="17" t="inlineStr">
@@ -2024,17 +2028,17 @@
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="B61" s="17" t="inlineStr">
         <is>
-          <t>An Excel worksheet laid out for Solver, with decision-variable cells, a SUMPRODUCT objective, and constraint formulas.</t>
+          <t>From constraints to the dual: every feasible y certifies an upper bound on profit, and the dual LP finds the best certificate.</t>
         </is>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>An Excel spreadsheet setup for a linear programming problem with decision variables in yellow cells. Constraints are defined with coefficients, totals, and right-hand side values.</t>
+          <t>Four-step flowchart deriving the dual: start with the primal constraints x1+x2&lt;=4 (flour) and 2x1+x2&lt;=5 (sugar); multiply by y1, y2 &gt;= 0 and add them into one inequality; choose y so the left side dominates the profit 3x1+2x2, giving the certificate 3x1+2x2 &lt;= 4y1+5y2; finally minimize the bound over all valid y, producing the dual LP: min 4y1+5y2 subject to y1+2y2&gt;=3, y1+y2&gt;=2, y&gt;=0.</t>
         </is>
       </c>
       <c r="D61" s="17" t="inlineStr">
@@ -2050,17 +2054,17 @@
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="B62" s="17" t="inlineStr">
         <is>
-          <t>The Solver sensitivity report: variable cells (final value, reduced cost, objective coefficient, allowable increase/decrease) and constraints (final value, shadow price, RHS, allowable increase/decrease).</t>
+          <t>Inventory risk cost as a function of inventory level.</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>A Microsoft Excel Solver sensitivity analysis report showing Variable Cells and Constraints sections with columns for Final Value, Reduced Cost, and Shadow Price.</t>
+          <t>Plot of the inventory risk function r(s) = c_r(1 - exp(-beta*s)) versus inventory level s: a smooth concave curve rising sharply from zero and saturating toward the maximum risk cost c_r, illustrating that marginal risk diminishes as inventory grows.</t>
         </is>
       </c>
       <c r="D62" s="17" t="inlineStr">
@@ -2076,17 +2080,17 @@
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="B63" s="17" t="inlineStr">
         <is>
-          <t>From constraints to the dual: every feasible y certifies an upper bound on profit, and the dual LP finds the best certificate.</t>
+          <t>Trade-off between total cost and maximum inventory risk.</t>
         </is>
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
-          <t>Four-step flowchart deriving the dual: start with the primal constraints x1+x2&lt;=4 (flour) and 2x1+x2&lt;=5 (sugar); multiply by y1, y2 &gt;= 0 and add them into one inequality; choose y so the left side dominates the profit 3x1+2x2, giving the certificate 3x1+2x2 &lt;= 4y1+5y2; finally minimize the bound over all valid y, producing the dual LP: min 4y1+5y2 subject to y1+2y2&gt;=3, y1+y2&gt;=2, y&gt;=0.</t>
+          <t>Pareto frontier curve for the multi-objective inventory problem, plotting total cost (horizontal axis) against maximum inventory risk (vertical axis). The downward-sloping non-dominated trade-off curve shows that lower risk can only be achieved by accepting higher cost.</t>
         </is>
       </c>
       <c r="D63" s="17" t="inlineStr">
@@ -2102,17 +2106,17 @@
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="B64" s="17" t="inlineStr">
         <is>
-          <t>Inventory risk cost as a function of inventory level.</t>
+          <t>Feasible region for the furniture production problem.</t>
         </is>
       </c>
       <c r="C64" s="17" t="inlineStr">
         <is>
-          <t>Plot of the inventory risk function r(s) = c_r(1 - exp(-beta*s)) versus inventory level s: a smooth concave curve rising sharply from zero and saturating toward the maximum risk cost c_r, illustrating that marginal risk diminishes as inventory grows.</t>
+          <t>Shaded feasible region in the plane of tables (x) and chairs (y), bounded by two blue constraint lines that intersect near (10, 8), with intercepts at 20 chairs and 12 tables.</t>
         </is>
       </c>
       <c r="D64" s="17" t="inlineStr">
@@ -2128,17 +2132,17 @@
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>13.4</t>
         </is>
       </c>
       <c r="B65" s="17" t="inlineStr">
         <is>
-          <t>Trade-off between total cost and maximum inventory risk.</t>
+          <t>Feasible set with revenue constrained to at least 70% of the maximum.</t>
         </is>
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
-          <t>Pareto frontier curve for the multi-objective inventory problem, plotting total cost (horizontal axis) against maximum inventory risk (vertical axis). The downward-sloping non-dominated trade-off curve shows that lower risk can only be achieved by accepting higher cost.</t>
+          <t>The furniture feasible region with red dashed revenue level lines and a darker shaded strip along the upper-right boundary marking the plans whose revenue is at least 70 percent of the maximum.</t>
         </is>
       </c>
       <c r="D65" s="17" t="inlineStr">
@@ -2154,17 +2158,17 @@
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="B66" s="17" t="inlineStr">
         <is>
-          <t>Feasible region for the furniture production problem.</t>
+          <t>The furniture problem in objective space: each point is a production plan (x,y) plotted by its revenue f1 (maximize) and rosewood waste f2 (minimize). The blue points are non-dominated: no feasible plan earns more revenue without creating more waste, and none creates less waste without giving up revenue. The red points are dominated; for example, (12,0) earns the same $96,000 as (10,8) but wastes 120 bdft instead of 116, and (4,4) matches the revenue of (0,20) with more waste. The frontier consists of the plans along x = 0 and along the rosewood constraint from (0,20) to (10,8).</t>
         </is>
       </c>
       <c r="C66" s="17" t="inlineStr">
         <is>
-          <t>Shaded feasible region in the plane of tables (x) and chairs (y), bounded by two blue constraint lines that intersect near (10, 8), with intercepts at 20 chairs and 12 tables.</t>
+          <t>Objective-space plot of rosewood waste f2=10x+2y against revenue f1=8000x+2000y (in thousands of dollars). Blue dots connected by a line mark Pareto optimal plans (the Pareto frontier); red squares lying above the line mark dominated plans, each labeled with its production plan (x, y).</t>
         </is>
       </c>
       <c r="D66" s="17" t="inlineStr">
@@ -2180,163 +2184,171 @@
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
         <is>
-          <t>13.4</t>
+          <t>14.1</t>
         </is>
       </c>
       <c r="B67" s="17" t="inlineStr">
         <is>
-          <t>Feasible set with revenue constrained to at least 70% of the maximum.</t>
+          <t>Aerial photograph of a Missoula, Montana housing development showing several blocks of houses...</t>
         </is>
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
-          <t>The furniture feasible region with red dashed revenue level lines and a darker shaded strip along the upper-right boundary marking the plans whose revenue is at least 70 percent of the maximum.</t>
+          <t>Aerial photograph of a Missoula, Montana housing development showing several blocks of houses connected by a network of streets. The image motivates the question of whether a lawn inspector can walk every street without backtracking.</t>
         </is>
       </c>
       <c r="D67" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E67" s="17" t="inlineStr"/>
-      <c r="F67" s="17" t="inlineStr"/>
+          <t>CC BY-SA 3.0; CC BY</t>
+        </is>
+      </c>
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society; aerial base image by Sam Beebe: Graphpicture</t>
+        </is>
+      </c>
+      <c r="F67" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society; aerial base image by Sam Beebe, "Graphpicture", CC BY-SA 3.0; CC BY</t>
+        </is>
+      </c>
       <c r="G67" s="17" t="inlineStr"/>
       <c r="H67" s="17" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>The furniture problem in objective space: each point is a production plan (x,y) plotted by its revenue f1 (maximize) and rosewood waste f2 (minimize). The blue points are non-dominated: no feasible plan earns more revenue without creating more waste, and none creates less waste without giving up revenue. The red points are dominated; for example, (12,0) earns the same $96,000 as (10,8) but wastes 120 bdft instead of 116, and (4,4) matches the revenue of (0,20) with more waste. The frontier consists of the plans along x = 0 and along the rosewood constraint from (0,20) to (10,8).</t>
+          <t>Side-by-side: the housing aerial photo is overlaid with red dots at intersections and red lines...</t>
         </is>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
-          <t>Objective-space plot of rosewood waste f2=10x+2y against revenue f1=8000x+2000y (in thousands of dollars). Blue dots connected by a line mark Pareto optimal plans (the Pareto frontier); red squares lying above the line mark dominated plans, each labeled with its production plan (x, y).</t>
+          <t>Side-by-side: the housing aerial photo is overlaid with red dots at intersections and red lines along streets; next to it, the same network is redrawn as a graph of labeled vertices joined by edges, showing the reduction of a street map to a graph.</t>
         </is>
       </c>
       <c r="D68" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E68" s="17" t="inlineStr"/>
-      <c r="F68" s="17" t="inlineStr"/>
+          <t>CC BY-SA 3.0; CC BY</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society; aerial base image by Sam Beebe: Graphpicturedot</t>
+        </is>
+      </c>
+      <c r="F68" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society; aerial base image by Sam Beebe, "Graphpicturedot", CC BY-SA 3.0; CC BY</t>
+        </is>
+      </c>
       <c r="G68" s="17" t="inlineStr"/>
       <c r="H68" s="17" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="B69" s="17" t="inlineStr">
         <is>
-          <t>Aerial photograph of a Missoula, Montana housing development showing several blocks of houses...</t>
+          <t>Eighteen-vertex housing-development graph with nodes A through R laid out on a roughly grid-like...</t>
         </is>
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
-          <t>Aerial photograph of a Missoula, Montana housing development showing several blocks of houses connected by a network of streets. The image motivates the question of whether a lawn inspector can walk every street without backtracking.</t>
+          <t>Eighteen-vertex housing-development graph with nodes A through R laid out on a roughly grid-like map of streets; reused from earlier in the chapter to ask whether an Euler circuit exists for the lawn inspector.</t>
         </is>
       </c>
       <c r="D69" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 3.0; CC BY</t>
-        </is>
-      </c>
-      <c r="E69" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society; aerial base image by Sam Beebe: Graphpicture</t>
-        </is>
-      </c>
-      <c r="F69" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society; aerial base image by Sam Beebe, "Graphpicture", CC BY-SA 3.0; CC BY</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr"/>
+      <c r="F69" s="17" t="inlineStr"/>
       <c r="G69" s="17" t="inlineStr"/>
       <c r="H69" s="17" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>14.4</t>
         </is>
       </c>
       <c r="B70" s="17" t="inlineStr">
         <is>
-          <t>Side-by-side: the housing aerial photo is overlaid with red dots at intersections and red lines...</t>
+          <t>The same 18-vertex graph G (vertices A through R) redrawn with vertices scattered in a non-grid layout.</t>
         </is>
       </c>
       <c r="C70" s="17" t="inlineStr">
         <is>
-          <t>Side-by-side: the housing aerial photo is overlaid with red dots at intersections and red lines along streets; next to it, the same network is redrawn as a graph of labeled vertices joined by edges, showing the reduction of a street map to a graph.</t>
+          <t>The same 18-vertex graph G (vertices A through R) redrawn with vertices scattered in a non-grid layout. The edge set is identical to the previous figure, illustrating that a graph's structure is independent of how it is drawn.</t>
         </is>
       </c>
       <c r="D70" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 3.0; CC BY</t>
-        </is>
-      </c>
-      <c r="E70" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society; aerial base image by Sam Beebe: Graphpicturedot</t>
-        </is>
-      </c>
-      <c r="F70" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society; aerial base image by Sam Beebe, "Graphpicturedot", CC BY-SA 3.0; CC BY</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="inlineStr"/>
+      <c r="F70" s="17" t="inlineStr"/>
       <c r="G70" s="17" t="inlineStr"/>
       <c r="H70" s="17" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="16" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="B71" s="17" t="inlineStr">
         <is>
-          <t>Eighteen-vertex housing-development graph with nodes A through R laid out on a roughly grid-like...</t>
+          <t>Historical map of the Prussian city of Koenigsberg with the river highlighted in blue and the seven...</t>
         </is>
       </c>
       <c r="C71" s="17" t="inlineStr">
         <is>
-          <t>Eighteen-vertex housing-development graph with nodes A through R laid out on a roughly grid-like map of streets; reused from earlier in the chapter to ask whether an Euler circuit exists for the lawn inspector.</t>
+          <t>Historical map of the Prussian city of Koenigsberg with the river highlighted in blue and the seven bridges that cross its forks marked in green, depicting the geographic setting of the famous Koenigsberg bridge problem that launched graph theory.</t>
         </is>
       </c>
       <c r="D71" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E71" s="17" t="inlineStr"/>
-      <c r="F71" s="17" t="inlineStr"/>
+          <t>CC BY-SA 3.0</t>
+        </is>
+      </c>
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>Bogdan Giusca, via Wikimedia Commons: Konigsberg Bridges</t>
+        </is>
+      </c>
+      <c r="F71" s="17" t="inlineStr">
+        <is>
+          <t>Bogdan Giusca, via Wikimedia Commons, "Konigsberg Bridges", CC BY-SA 3.0, https://commons.wikimedia.org/wiki/File:Konigsberg_bridges.png</t>
+        </is>
+      </c>
       <c r="G71" s="17" t="inlineStr"/>
       <c r="H71" s="17" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
-          <t>14.4</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>The same 18-vertex graph G (vertices A through R) redrawn with vertices scattered in a non-grid layout.</t>
+          <t>Schematic of Konigsberg’s four landmasses drawn as labelled ellipses (North Bank, Island, East...</t>
         </is>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
-          <t>The same 18-vertex graph G (vertices A through R) redrawn with vertices scattered in a non-grid layout. The edge set is identical to the previous figure, illustrating that a graph's structure is independent of how it is drawn.</t>
+          <t>Schematic of Konigsberg's four landmasses drawn as labelled ellipses (North Bank, Island, East Bank, South Bank) with seven short line segments crossing between them representing the seven bridges of the puzzle.</t>
         </is>
       </c>
       <c r="D72" s="17" t="inlineStr">
@@ -2352,51 +2364,43 @@
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
         <is>
-          <t>14.5</t>
+          <t>14.7</t>
         </is>
       </c>
       <c r="B73" s="17" t="inlineStr">
         <is>
-          <t>Historical map of the Prussian city of Koenigsberg with the river highlighted in blue and the seven...</t>
+          <t>Graph abstraction of the Konigsberg bridges: four circular vertices labelled NB, I, EB, and SB with...</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
         <is>
-          <t>Historical map of the Prussian city of Koenigsberg with the river highlighted in blue and the seven bridges that cross its forks marked in green, depicting the geographic setting of the famous Koenigsberg bridge problem that launched graph theory.</t>
+          <t>Graph abstraction of the Konigsberg bridges: four circular vertices labelled NB, I, EB, and SB with seven edges connecting them, including two parallel arcs between NB and I and two between I and SB to represent the duplicate bridges (a multigraph).</t>
         </is>
       </c>
       <c r="D73" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 3.0</t>
-        </is>
-      </c>
-      <c r="E73" s="17" t="inlineStr">
-        <is>
-          <t>Bogdan Giusca, via Wikimedia Commons: Konigsberg Bridges</t>
-        </is>
-      </c>
-      <c r="F73" s="17" t="inlineStr">
-        <is>
-          <t>Bogdan Giusca, via Wikimedia Commons, "Konigsberg Bridges", CC BY-SA 3.0, https://commons.wikimedia.org/wiki/File:Konigsberg_bridges.png</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E73" s="17" t="inlineStr"/>
+      <c r="F73" s="17" t="inlineStr"/>
       <c r="G73" s="17" t="inlineStr"/>
       <c r="H73" s="17" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>14.8</t>
         </is>
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>Schematic of Konigsberg’s four landmasses drawn as labelled ellipses (North Bank, Island, East...</t>
+          <t>Small graph illustrating a loop: three filled-dot vertices form a triangle and a red self-loop...</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>Schematic of Konigsberg's four landmasses drawn as labelled ellipses (North Bank, Island, East Bank, South Bank) with seven short line segments crossing between them representing the seven bridges of the puzzle.</t>
+          <t>Small graph illustrating a loop: three filled-dot vertices form a triangle and a red self-loop attaches to the rightmost vertex, showing an edge that connects a vertex to itself.</t>
         </is>
       </c>
       <c r="D74" s="17" t="inlineStr">
@@ -2412,67 +2416,15 @@
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
         <is>
-          <t>14.7</t>
+          <t>14.9</t>
         </is>
       </c>
       <c r="B75" s="17" t="inlineStr">
         <is>
-          <t>Graph abstraction of the Konigsberg bridges: four circular vertices labelled NB, I, EB, and SB with...</t>
+          <t>Examples of vertices of degree 0 through 4.</t>
         </is>
       </c>
       <c r="C75" s="17" t="inlineStr">
-        <is>
-          <t>Graph abstraction of the Konigsberg bridges: four circular vertices labelled NB, I, EB, and SB with seven edges connecting them, including two parallel arcs between NB and I and two between I and SB to represent the duplicate bridges (a multigraph).</t>
-        </is>
-      </c>
-      <c r="D75" s="17" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E75" s="17" t="inlineStr"/>
-      <c r="F75" s="17" t="inlineStr"/>
-      <c r="G75" s="17" t="inlineStr"/>
-      <c r="H75" s="17" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="16" t="inlineStr">
-        <is>
-          <t>14.8</t>
-        </is>
-      </c>
-      <c r="B76" s="17" t="inlineStr">
-        <is>
-          <t>Small graph illustrating a loop: three filled-dot vertices form a triangle and a red self-loop...</t>
-        </is>
-      </c>
-      <c r="C76" s="17" t="inlineStr">
-        <is>
-          <t>Small graph illustrating a loop: three filled-dot vertices form a triangle and a red self-loop attaches to the rightmost vertex, showing an edge that connects a vertex to itself.</t>
-        </is>
-      </c>
-      <c r="D76" s="17" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E76" s="17" t="inlineStr"/>
-      <c r="F76" s="17" t="inlineStr"/>
-      <c r="G76" s="17" t="inlineStr"/>
-      <c r="H76" s="17" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="16" t="inlineStr">
-        <is>
-          <t>14.9</t>
-        </is>
-      </c>
-      <c r="B77" s="17" t="inlineStr">
-        <is>
-          <t>Examples of vertices of degree 0 through 4.</t>
-        </is>
-      </c>
-      <c r="C77" s="17" t="inlineStr">
         <is>
           <t>Single isolated vertex with no edges, illustrating a vertex of degree 0 in the table of degree examples.
 A vertex with one edge attached, illustrating degree 1 in the table of degree examples.
@@ -2481,6 +2433,58 @@
 A vertex with four edges attached (one to each diagonal direction), illustrating degree 4 in the table of degree examples.</t>
         </is>
       </c>
+      <c r="D75" s="17" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E75" s="17" t="inlineStr"/>
+      <c r="F75" s="17" t="inlineStr"/>
+      <c r="G75" s="17" t="inlineStr"/>
+      <c r="H75" s="17" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>14.10</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="inlineStr">
+        <is>
+          <t>A 3-by-4 grid graph with 12 vertices labelled A-D (top), E-H (middle), J-M (bottom).</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t>A 3-by-4 grid graph with 12 vertices labelled A-D (top), E-H (middle), J-M (bottom). All grid edges are drawn; a path from A to M is highlighted in thick red, traversing A-E-F-G-L-M.</t>
+        </is>
+      </c>
+      <c r="D76" s="17" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E76" s="17" t="inlineStr"/>
+      <c r="F76" s="17" t="inlineStr"/>
+      <c r="G76" s="17" t="inlineStr"/>
+      <c r="H76" s="17" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>14.11</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="inlineStr">
+        <is>
+          <t>The same 3-by-4 grid graph (vertices A-D, E-H, J-M) with a circuit highlighted in thick red...</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>The same 3-by-4 grid graph (vertices A-D, E-H, J-M) with a circuit highlighted in thick red, beginning and ending at vertex A by traversing A-E-J-K-F-B-A and similar back path, illustrating a cycle.</t>
+        </is>
+      </c>
       <c r="D77" s="17" t="inlineStr">
         <is>
           <t>CC BY-SA 4.0 (original figure created for this book)</t>
@@ -2494,17 +2498,17 @@
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
         <is>
-          <t>14.10</t>
+          <t>14.12</t>
         </is>
       </c>
       <c r="B78" s="17" t="inlineStr">
         <is>
-          <t>A 3-by-4 grid graph with 12 vertices labelled A-D (top), E-H (middle), J-M (bottom).</t>
+          <t>A 3-by-4 grid graph with vertices A-D, E-H, J-M, but with the column-A horizontal edges deleted so...</t>
         </is>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
-          <t>A 3-by-4 grid graph with 12 vertices labelled A-D (top), E-H (middle), J-M (bottom). All grid edges are drawn; a path from A to M is highlighted in thick red, traversing A-E-F-G-L-M.</t>
+          <t>A 3-by-4 grid graph with vertices A-D, E-H, J-M, but with the column-A horizontal edges deleted so that vertex A and the left column are isolated from the rest, illustrating a disconnected graph.</t>
         </is>
       </c>
       <c r="D78" s="17" t="inlineStr">
@@ -2520,17 +2524,17 @@
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
         <is>
-          <t>14.11</t>
+          <t>14.13</t>
         </is>
       </c>
       <c r="B79" s="17" t="inlineStr">
         <is>
-          <t>The same 3-by-4 grid graph (vertices A-D, E-H, J-M) with a circuit highlighted in thick red...</t>
+          <t>Weighted graph of five U.S. cities (LA, Seattle, Chicago, Atlanta, Dallas) shown as filled dots...</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
-          <t>The same 3-by-4 grid graph (vertices A-D, E-H, J-M) with a circuit highlighted in thick red, beginning and ending at vertex A by traversing A-E-J-K-F-B-A and similar back path, illustrating a cycle.</t>
+          <t>Weighted graph of five U.S. cities (LA, Seattle, Chicago, Atlanta, Dallas) shown as filled dots arranged across the plane, with all ten edges drawn and labelled with one-way airfares such as $70 (LA-Seattle), $150 (LA-Dallas), $85 (Atlanta-Dallas), $75 (Chicago-Atlanta).</t>
         </is>
       </c>
       <c r="D79" s="17" t="inlineStr">
@@ -2546,17 +2550,18 @@
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
         <is>
-          <t>14.12</t>
+          <t>14.14</t>
         </is>
       </c>
       <c r="B80" s="17" t="inlineStr">
         <is>
-          <t>A 3-by-4 grid graph with vertices A-D, E-H, J-M, but with the column-A horizontal edges deleted so...</t>
+          <t>Weighted road network for the Yakima-to-Tacoma example: seven filled-dot vertices T (Tacoma), E...</t>
         </is>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
-          <t>A 3-by-4 grid graph with vertices A-D, E-H, J-M, but with the column-A horizontal edges deleted so that vertex A and the left column are isolated from the rest, illustrating a disconnected graph.</t>
+          <t>PIC
+Weighted road network for the Yakima-to-Tacoma example: seven filled-dot vertices T (Tacoma), E (Eatonville), A (Auburn), NB (North Bend), MR (Mount Rainier), P (Packwood), Y (Yakima) with edges labelled by travel times in minutes (e.g., T-A=20, A-NB=36, NB-Y=104, MR-Y=96, P-Y=76).</t>
         </is>
       </c>
       <c r="D80" s="17" t="inlineStr">
@@ -2572,17 +2577,17 @@
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
         <is>
-          <t>14.13</t>
+          <t>14.15</t>
         </is>
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>Weighted graph of five U.S. cities (LA, Seattle, Chicago, Atlanta, Dallas) shown as filled dots...</t>
+          <t>Yakima-to-Tacoma road network as before, now with the destination Y annotated [0] in red to mark it...</t>
         </is>
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>Weighted graph of five U.S. cities (LA, Seattle, Chicago, Atlanta, Dallas) shown as filled dots arranged across the plane, with all ten edges drawn and labelled with one-way airfares such as $70 (LA-Seattle), $150 (LA-Dallas), $85 (Atlanta-Dallas), $75 (Chicago-Atlanta).</t>
+          <t>Yakima-to-Tacoma road network as before, now with the destination Y annotated [0] in red to mark it as the starting vertex of Dijkstra's algorithm with tentative distance zero.</t>
         </is>
       </c>
       <c r="D81" s="17" t="inlineStr">
@@ -2598,18 +2603,17 @@
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
         <is>
-          <t>14.14</t>
+          <t>14.16</t>
         </is>
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>Weighted road network for the Yakima-to-Tacoma example: seven filled-dot vertices T (Tacoma), E...</t>
+          <t>Yakima example after Dijkstra step 2: tentative distances [104] at NB, [96] at MR, [76] at P are...</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
-          <t>Initial-state diagram for Dijkstra's algorithm: seven blue circular nodes T, E, A, NB, MR, P, Y connected by weighted edges (e.g., T-A=20, A-NB=36, NB-Y=120, MR-Y=90); each node has a green-boxed tentative-distance label, all set to infinity except the destination T which is 0.
-Weighted road network for the Yakima-to-Tacoma example: seven filled-dot vertices T (Tacoma), E (Eatonville), A (Auburn), NB (North Bend), MR (Mount Rainier), P (Packwood), Y (Yakima) with edges labelled by travel times in minutes (e.g., T-A=20, A-NB=36, NB-Y=104, MR-Y=96, P-Y=76).</t>
+          <t>Yakima example after Dijkstra step 2: tentative distances [104] at NB, [96] at MR, [76] at P are recorded in red next to each neighbour of Y; Y still labelled [0]; remaining vertices T, E, A are unlabelled.</t>
         </is>
       </c>
       <c r="D82" s="17" t="inlineStr">
@@ -2625,17 +2629,17 @@
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
         <is>
-          <t>14.15</t>
+          <t>14.17</t>
         </is>
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>Yakima-to-Tacoma road network as before, now with the destination Y annotated [0] in red to mark it...</t>
+          <t>Yakima example after the second iteration: P is the current vertex; E now has tentative distance...</t>
         </is>
       </c>
       <c r="C83" s="17" t="inlineStr">
         <is>
-          <t>Yakima-to-Tacoma road network as before, now with the destination Y annotated [0] in red to mark it as the starting vertex of Dijkstra's algorithm with tentative distance zero.</t>
+          <t>Yakima example after the second iteration: P is the current vertex; E now has tentative distance [172] (via P), and Y is shown struck-through (visited); other labels [104] at NB, [96] at MR, [76] at P remain.</t>
         </is>
       </c>
       <c r="D83" s="17" t="inlineStr">
@@ -2651,17 +2655,17 @@
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
         <is>
-          <t>14.16</t>
+          <t>14.18</t>
         </is>
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after Dijkstra step 2: tentative distances [104] at NB, [96] at MR, [76] at P are...</t>
+          <t>Yakima example after the third iteration: A has tentative distance [175] (via MR); P and Y appear...</t>
         </is>
       </c>
       <c r="C84" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after Dijkstra step 2: tentative distances [104] at NB, [96] at MR, [76] at P are recorded in red next to each neighbour of Y; Y still labelled [0]; remaining vertices T, E, A are unlabelled.</t>
+          <t>Yakima example after the third iteration: A has tentative distance [175] (via MR); P and Y appear struck-through (visited); NB still [104], MR [96], E [172].</t>
         </is>
       </c>
       <c r="D84" s="17" t="inlineStr">
@@ -2677,17 +2681,17 @@
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
         <is>
-          <t>14.17</t>
+          <t>14.19</t>
         </is>
       </c>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the second iteration: P is the current vertex; E now has tentative distance...</t>
+          <t>Yakima example after the fourth iteration: A’s distance is updated to [140] via NB; NB, MR, P, Y...</t>
         </is>
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the second iteration: P is the current vertex; E now has tentative distance [172] (via P), and Y is shown struck-through (visited); other labels [104] at NB, [96] at MR, [76] at P remain.</t>
+          <t>Yakima example after the fourth iteration: A's distance is updated to [140] via NB; NB, MR, P, Y all struck-through; E still [172].</t>
         </is>
       </c>
       <c r="D85" s="17" t="inlineStr">
@@ -2703,17 +2707,17 @@
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
         <is>
-          <t>14.18</t>
+          <t>14.20</t>
         </is>
       </c>
       <c r="B86" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the third iteration: A has tentative distance [175] (via MR); P and Y appear...</t>
+          <t>Yakima example after the fifth iteration: T receives tentative distance [160] via A; A, NB, MR, P...</t>
         </is>
       </c>
       <c r="C86" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the third iteration: A has tentative distance [175] (via MR); P and Y appear struck-through (visited); NB still [104], MR [96], E [172].</t>
+          <t>Yakima example after the fifth iteration: T receives tentative distance [160] via A; A, NB, MR, P, Y are struck-through, leaving E [172] still active. The shortest path T-A-NB-Y of 160 minutes is now determined.</t>
         </is>
       </c>
       <c r="D86" s="17" t="inlineStr">
@@ -2729,17 +2733,17 @@
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>14.21</t>
         </is>
       </c>
       <c r="B87" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the fourth iteration: A’s distance is updated to [140] via NB; NB, MR, P, Y...</t>
+          <t>Weighted undirected graph for the Dijkstra example.</t>
         </is>
       </c>
       <c r="C87" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the fourth iteration: A's distance is updated to [140] via NB; NB, MR, P, Y all struck-through; E still [172].</t>
+          <t>Weighted undirected graph for the Dijkstra example. Seven vertices a-g are joined by edges with weights a-b=2, a-c=6, c-d=8, b-d=5, d-e=10, d-f=15, e-f=6, e-g=2, f-g=6. No vertex is yet marked visited.</t>
         </is>
       </c>
       <c r="D87" s="17" t="inlineStr">
@@ -2755,17 +2759,17 @@
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
         <is>
-          <t>14.20</t>
+          <t>14.22</t>
         </is>
       </c>
       <c r="B88" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the fifth iteration: T receives tentative distance [160] via A; A, NB, MR, P...</t>
+          <t>Dijkstra step 1: the start vertex a is highlighted in red and labeled with tentative distance 0.</t>
         </is>
       </c>
       <c r="C88" s="17" t="inlineStr">
         <is>
-          <t>Yakima example after the fifth iteration: T receives tentative distance [160] via A; A, NB, MR, P, Y are struck-through, leaving E [172] still active. The shortest path Y-NB-A-T of 160 minutes is now determined.</t>
+          <t>Dijkstra step 1: the start vertex a is highlighted in red and labeled with tentative distance 0. Its neighbors b and c receive tentative labels 2 and 6 from a; all other vertices remain labeled infinity.</t>
         </is>
       </c>
       <c r="D88" s="17" t="inlineStr">
@@ -2781,17 +2785,17 @@
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
         <is>
-          <t>14.21</t>
+          <t>14.23</t>
         </is>
       </c>
       <c r="B89" s="17" t="inlineStr">
         <is>
-          <t>Weighted undirected graph for the Dijkstra example.</t>
+          <t>Dijkstra step 2: vertex b is now marked as visited with permanent distance 2, and the edge a-b is...</t>
         </is>
       </c>
       <c r="C89" s="17" t="inlineStr">
         <is>
-          <t>Weighted undirected graph for the Dijkstra example. Seven vertices a-g are joined by edges with weights a-b=2, a-c=6, c-d=8, b-d=5, d-e=10, d-f=15, e-f=6, e-g=2, f-g=6. No vertex is yet marked visited.</t>
+          <t>Dijkstra step 2: vertex b is now marked as visited with permanent distance 2, and the edge a-b is highlighted in red. Vertex d is updated through b to tentative distance 7. Labels at c, e, f, and g are unchanged.</t>
         </is>
       </c>
       <c r="D89" s="17" t="inlineStr">
@@ -2807,17 +2811,17 @@
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
         <is>
-          <t>14.22</t>
+          <t>14.24</t>
         </is>
       </c>
       <c r="B90" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 1: the start vertex a is highlighted in red and labeled with tentative distance 0.</t>
+          <t>Dijkstra step 3: vertex c is marked visited with distance 6 and edge a-c is highlighted.</t>
         </is>
       </c>
       <c r="C90" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 1: the start vertex a is highlighted in red and labeled with tentative distance 0. Its neighbors b and c receive tentative labels 2 and 6 from a; all other vertices remain labeled infinity.</t>
+          <t>Dijkstra step 3: vertex c is marked visited with distance 6 and edge a-c is highlighted. Reaching d through c would give 6+8=14, which is worse than the current label 7, so d's tentative distance is unchanged.</t>
         </is>
       </c>
       <c r="D90" s="17" t="inlineStr">
@@ -2833,17 +2837,17 @@
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
         <is>
-          <t>14.23</t>
+          <t>14.25</t>
         </is>
       </c>
       <c r="B91" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 2: vertex b is now marked as visited with permanent distance 2, and the edge a-b is...</t>
+          <t>Dijkstra step 4: vertex d is marked visited with distance 7, and the path a-b-d is highlighted in red.</t>
         </is>
       </c>
       <c r="C91" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 2: vertex b is now marked as visited with permanent distance 2, and the edge a-b is highlighted in red. Vertex d is updated through b to tentative distance 7. Labels at c, e, f, and g are unchanged.</t>
+          <t>Dijkstra step 4: vertex d is marked visited with distance 7, and the path a-b-d is highlighted in red. Neighbors of d are updated: e to 17 (via 7+10) and f to 22 (via 7+15); g remains infinity.</t>
         </is>
       </c>
       <c r="D91" s="17" t="inlineStr">
@@ -2859,17 +2863,17 @@
     <row r="92">
       <c r="A92" s="16" t="inlineStr">
         <is>
-          <t>14.24</t>
+          <t>14.26</t>
         </is>
       </c>
       <c r="B92" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 3: vertex c is marked visited with distance 6 and edge a-c is highlighted.</t>
+          <t>Dijkstra step 5: vertex e is marked visited with distance 17 and the edge d-e is added to the...</t>
         </is>
       </c>
       <c r="C92" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 3: vertex c is marked visited with distance 6 and edge a-c is highlighted. Reaching d through c would give 6+8=14, which is worse than the current label 7, so d's tentative distance is unchanged.</t>
+          <t>Dijkstra step 5: vertex e is marked visited with distance 17 and the edge d-e is added to the highlighted path. From e, vertex g is updated to 17+2=19, improving on its previous infinity label.</t>
         </is>
       </c>
       <c r="D92" s="17" t="inlineStr">
@@ -2885,17 +2889,17 @@
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
         <is>
-          <t>14.25</t>
+          <t>14.27</t>
         </is>
       </c>
       <c r="B93" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 4: vertex d is marked visited with distance 7, and the path a-b-d is highlighted in red.</t>
+          <t>Dijkstra step 6: vertex g is marked visited with distance 19, and the edge e-g is highlighted...</t>
         </is>
       </c>
       <c r="C93" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 4: vertex d is marked visited with distance 7, and the path a-b-d is highlighted in red. Neighbors of d are updated: e to 17 (via 7+10) and f to 22 (via 7+15); g remains infinity.</t>
+          <t>Dijkstra step 6: vertex g is marked visited with distance 19, and the edge e-g is highlighted, completing a tentative shortest path a-b-d-e-g. The remaining unvisited vertex f keeps tentative distance 22.</t>
         </is>
       </c>
       <c r="D93" s="17" t="inlineStr">
@@ -2911,17 +2915,17 @@
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
         <is>
-          <t>14.26</t>
+          <t>14.28</t>
         </is>
       </c>
       <c r="B94" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 5: vertex e is marked visited with distance 17 and the edge d-e is added to the...</t>
+          <t>Dijkstra step 7: vertex f is marked visited with distance 22 and the edge d-f is highlighted along...</t>
         </is>
       </c>
       <c r="C94" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 5: vertex e is marked visited with distance 17 and the edge d-e is added to the highlighted path. From e, vertex g is updated to 17+2=19, improving on its previous infinity label.</t>
+          <t>Dijkstra step 7: vertex f is marked visited with distance 22 and the edge d-f is highlighted along with the previously found path. All seven vertices are now visited so the algorithm terminates.</t>
         </is>
       </c>
       <c r="D94" s="17" t="inlineStr">
@@ -2937,17 +2941,17 @@
     <row r="95">
       <c r="A95" s="16" t="inlineStr">
         <is>
-          <t>14.27</t>
+          <t>14.29</t>
         </is>
       </c>
       <c r="B95" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 6: vertex g is marked visited with distance 19, and the edge e-g is highlighted...</t>
+          <t>Final state of the Dijkstra example: every vertex carries its shortest-path distance from a (a=0...</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 6: vertex g is marked visited with distance 19, and the edge e-g is highlighted, completing a tentative shortest path a-b-d-e-g. The remaining unvisited vertex f keeps tentative distance 22.</t>
+          <t>Final state of the Dijkstra example: every vertex carries its shortest-path distance from a (a=0, b=2, c=6, d=7, e=17, g=19, f=22), and the shortest-path tree found by the algorithm is highlighted in red.</t>
         </is>
       </c>
       <c r="D95" s="17" t="inlineStr">
@@ -2963,17 +2967,17 @@
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
         <is>
-          <t>14.28</t>
+          <t>14.30</t>
         </is>
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 7: vertex f is marked visited with distance 22 and the edge d-f is highlighted along...</t>
+          <t>The same seven-vertex weighted graph with the shortest path from a to g highlighted in red...</t>
         </is>
       </c>
       <c r="C96" s="17" t="inlineStr">
         <is>
-          <t>Dijkstra step 7: vertex f is marked visited with distance 22 and the edge d-f is highlighted along with the previously found path. All seven vertices are now visited so the algorithm terminates.</t>
+          <t>The same seven-vertex weighted graph with the shortest path from a to g highlighted in red: a-b-d-e-g, traversing edges of weight 2, 5, 10, and 2 for a total length of 19.</t>
         </is>
       </c>
       <c r="D96" s="17" t="inlineStr">
@@ -2989,17 +2993,17 @@
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
         <is>
-          <t>14.29</t>
+          <t>14.31</t>
         </is>
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>Final state of the Dijkstra example: every vertex carries its shortest-path distance from a (a=0...</t>
+          <t>Weighted graph of leasing costs, in thousands of dollars per year, between the five offices A, B, C, D, E.</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
         <is>
-          <t>Final state of the Dijkstra example: every vertex carries its shortest-path distance from a (a=0, b=2, c=6, d=7, e=17, g=19, f=22), and the shortest-path tree found by the algorithm is highlighted in red.</t>
+          <t>A 4-vertex spanning tree drawn as filled dots at corners of a small region, connected by three edges forming a Y-shape (top-left to top vertex, bottom-right to middle, top to bottom-right), illustrating one possible spanning tree on four vertices.</t>
         </is>
       </c>
       <c r="D97" s="17" t="inlineStr">
@@ -3015,17 +3019,17 @@
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
         <is>
-          <t>14.30</t>
+          <t>14.32</t>
         </is>
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>The same seven-vertex weighted graph with the shortest path from a to g highlighted in red...</t>
+          <t>A spanning tree on four vertices with three edges.</t>
         </is>
       </c>
       <c r="C98" s="17" t="inlineStr">
         <is>
-          <t>The same seven-vertex weighted graph with the shortest path from a to g highlighted in red: a-b-d-e-g, traversing edges of weight 2, 5, 10, and 2 for a total length of 19.</t>
+          <t>A 4-vertex spanning tree with three edges arranged as a path: middle vertex linked to top-right, top-right linked to bottom-right, and bottom-right linked to bottom-left, showing another spanning-tree configuration on four vertices.</t>
         </is>
       </c>
       <c r="D98" s="17" t="inlineStr">
@@ -3041,17 +3045,17 @@
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
         <is>
-          <t>14.31</t>
+          <t>14.33</t>
         </is>
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>A 4-vertex spanning tree drawn as filled dots at corners of a small region, connected by three...</t>
+          <t>Another spanning tree on the same four vertices.</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
         <is>
-          <t>A 4-vertex spanning tree drawn as filled dots at corners of a small region, connected by three edges forming a Y-shape (top-left to top vertex, bottom-right to middle, top to bottom-right), illustrating one possible spanning tree on four vertices.</t>
+          <t>Composite figure of five small spanning trees with n = 1, 2, 3, 4, 5 vertices arranged left-to-right; each tree has exactly n-1 edges, demonstrating that a spanning tree on n vertices uses n-1 edges.</t>
         </is>
       </c>
       <c r="D99" s="17" t="inlineStr">
@@ -3067,17 +3071,20 @@
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
         <is>
-          <t>14.32</t>
+          <t>14.34</t>
         </is>
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>A 4-vertex spanning tree with three edges arranged as a path: middle vertex linked to top-right...</t>
+          <t>Examples of spanning trees with n = 1,2,3,4,5 nodes and exactly n − 1 edges</t>
         </is>
       </c>
       <c r="C100" s="17" t="inlineStr">
         <is>
-          <t>A 4-vertex spanning tree with three edges arranged as a path: middle vertex linked to top-right, top-right linked to bottom-right, and bottom-right linked to bottom-left, showing another spanning-tree configuration on four vertices.</t>
+          <t>n = 3 case from the spanning-tree examples: three labelled vertices A, B, C connected by two edges (A-B and B-C) forming a path, with exactly n-1 = 2 edges.
+n = 4 case from the spanning-tree examples: a star tree with center B connected to leaves A, C, and D by three edges, illustrating n-1 = 3 edges on n = 4 vertices.
+Five small spanning trees side by side on n = 1, 2, 3, 4, 5 vertices. Yellow circular nodes labelled A through E are connected by exactly n-1 edges in each, supporting the lemma that a tree on n vertices has n-1 edges.
+Single yellow circular node labelled A drawn in isolation, illustrating the base case of the induction proof: a tree with one vertex and zero edges satisfies |E| = n - 1 = 0.</t>
         </is>
       </c>
       <c r="D100" s="17" t="inlineStr">
@@ -3093,17 +3100,17 @@
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
         <is>
-          <t>14.33</t>
+          <t>14.35</t>
         </is>
       </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>Composite figure of five small spanning trees with n = 1, 2, 3, 4, 5 vertices arranged...</t>
+          <t>Base case: A single vertex with no edges</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
         <is>
-          <t>Composite figure of five small spanning trees with n = 1, 2, 3, 4, 5 vertices arranged left-to-right; each tree has exactly n-1 edges, demonstrating that a spanning tree on n vertices uses n-1 edges.</t>
+          <t>A single yellow vertex labeled A with no edges: the smallest possible graph.</t>
         </is>
       </c>
       <c r="D101" s="17" t="inlineStr">
@@ -3119,20 +3126,17 @@
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
         <is>
-          <t>14.34</t>
+          <t>14.36</t>
         </is>
       </c>
       <c r="B102" s="17" t="inlineStr">
         <is>
-          <t>Examples of spanning trees with n = 1,2,3,4,5 nodes and exactly n − 1 edges</t>
+          <t>Inductive step: Removing the leaf L and its dashed edge reduces the tree to 4 vertices and 3 edges</t>
         </is>
       </c>
       <c r="C102" s="17" t="inlineStr">
         <is>
-          <t>n = 3 case from the spanning-tree examples: three labelled vertices A, B, C connected by two edges (A-B and B-C) forming a path, with exactly n-1 = 2 edges.
-n = 4 case from the spanning-tree examples: a star tree with center B connected to leaves A, C, and D by three edges, illustrating n-1 = 3 edges on n = 4 vertices.
-Five small spanning trees side by side on n = 1, 2, 3, 4, 5 vertices. Yellow circular nodes labelled A through E are connected by exactly n-1 edges in each, supporting the lemma that a tree on n vertices has n-1 edges.
-Single yellow circular node labelled A drawn in isolation, illustrating the base case of the induction proof: a tree with one vertex and zero edges satisfies |E| = n - 1 = 0.</t>
+          <t>Pseudocode block titled 'Kruskal's Algorithm (Descriptive Version)'. Initialize T to empty; repeatedly pick the cheapest unused edge, skipping any edge that would create a cycle; stop once T contains |V|-1 edges, forming a minimum spanning tree of G.</t>
         </is>
       </c>
       <c r="D102" s="17" t="inlineStr">
@@ -3148,17 +3152,17 @@
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
         <is>
-          <t>14.35</t>
+          <t>14.37</t>
         </is>
       </c>
       <c r="B103" s="17" t="inlineStr">
         <is>
-          <t>Base case: A single vertex with no edges</t>
+          <t>Five-vertex graph with cities A, B, C, D, E as black dots, fully connected with dollar-cost edge...</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
         <is>
-          <t>A single yellow vertex labeled A with no edges: the smallest possible graph.</t>
+          <t>Five-vertex graph with cities A, B, C, D, E as black dots, fully connected with dollar-cost edge labels (AB=4, AE=5, AC=8, DC=7, plus higher cross-edges). Edges AB, AE, AC, DC are thick red, marking the MST built by Prim's algorithm starting at A.</t>
         </is>
       </c>
       <c r="D103" s="17" t="inlineStr">
@@ -3174,17 +3178,17 @@
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
         <is>
-          <t>14.36</t>
+          <t>14.38</t>
         </is>
       </c>
       <c r="B104" s="17" t="inlineStr">
         <is>
-          <t>Inductive step: Removing the leaf L and its dashed edge reduces the tree to 4 vertices and 3 edges</t>
+          <t>A spanning subgraph of the Oregon cities graph.</t>
         </is>
       </c>
       <c r="C104" s="17" t="inlineStr">
         <is>
-          <t>Pseudocode block titled 'Kruskal's Algorithm (Descriptive Version)'. Initialize T to empty; repeatedly pick the cheapest unused edge, skipping any edge that would create a cycle; stop once T contains |V|-1 edges, forming a minimum spanning tree of G.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D104" s="17" t="inlineStr">
@@ -3200,17 +3204,17 @@
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
         <is>
-          <t>14.37</t>
+          <t>14.39</t>
         </is>
       </c>
       <c r="B105" s="17" t="inlineStr">
         <is>
-          <t>Five-vertex graph with cities A, B, C, D, E as black dots, fully connected with dollar-cost edge...</t>
+          <t>Another subgraph of the Oregon cities graph.</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
         <is>
-          <t>Five-vertex graph with cities A, B, C, D, E as black dots, fully connected with dollar-cost edge labels (AB=4, AE=5, AC=8, DC=7, plus higher cross-edges). Edges AB, AE, AC, DC are thick red, marking the MST built by Prim's algorithm starting at A.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D105" s="17" t="inlineStr">
@@ -3226,17 +3230,17 @@
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
         <is>
-          <t>14.38</t>
+          <t>14.40</t>
         </is>
       </c>
       <c r="B106" s="17" t="inlineStr">
         <is>
-          <t>A spanning subgraph of the Oregon cities graph.</t>
+          <t>Undirected weighted graph with six yellow circular vertices A, B, C, E, F, G arranged hexagonally.</t>
         </is>
       </c>
       <c r="C106" s="17" t="inlineStr">
         <is>
-          <t>A spanning subgraph of the Oregon cities graph.</t>
+          <t>Undirected weighted graph with six yellow circular vertices A, B, C, E, F, G arranged hexagonally. Every pair is joined by an edge labelled with its integer weight (e.g. AB=11, BG=13, AE=14, EF=16, AC=33). Input graph for the Kruskal exercise.</t>
         </is>
       </c>
       <c r="D106" s="17" t="inlineStr">
@@ -3252,17 +3256,19 @@
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
         <is>
-          <t>14.39</t>
+          <t>14.41</t>
         </is>
       </c>
       <c r="B107" s="17" t="inlineStr">
         <is>
-          <t>Another subgraph of the Oregon cities graph.</t>
+          <t>Prim’s algorithm</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
         <is>
-          <t>Another subgraph of the Oregon cities graph.</t>
+          <t>Python code listing 'Loading the graph into NetworkX' that builds the prior 6-vertex weighted graph in NetworkX: it imports nx, creates an undirected Graph, adds nodes A,B,C,E,F,G, and feeds the 15 weighted edges via G.add_weighted_edges_from(edges).
+Five-vertex graph with cities A, B, C, D, E as black dots, fully connected with dollar-cost edge labels (AB=4, AE=5, AC=8, DC=7, plus higher cross-edges). Edges AB, AE, AC, DC are thick red, marking the MST built by Prim's algorithm starting at A.
+Same five-city phone-line graph (A, B, C, D, E) used to illustrate Prim's algorithm. Edges are labelled with dollar costs and the spanning tree edges AB, AE, AC, DC are drawn in thick red while the remaining inter-city edges are thin black.</t>
         </is>
       </c>
       <c r="D107" s="17" t="inlineStr">
@@ -3278,17 +3284,17 @@
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
         <is>
-          <t>14.40</t>
+          <t>14.42</t>
         </is>
       </c>
       <c r="B108" s="17" t="inlineStr">
         <is>
-          <t>Undirected weighted graph with six yellow circular vertices A, B, C, E, F, G arranged hexagonally.</t>
+          <t>Weighted graph with seven vertices A through G for the shortest path exercise.</t>
         </is>
       </c>
       <c r="C108" s="17" t="inlineStr">
         <is>
-          <t>Undirected weighted graph with six yellow circular vertices A, B, C, E, F, G arranged hexagonally. Every pair is joined by an edge labelled with its integer weight (e.g. AB=11, BG=13, AE=14, EF=16, AC=33). Input graph for the Kruskal exercise.</t>
+          <t>Boxed figure for Prim's algorithm: 7-vertex graph with vertices a, b, c, d, e, f, g as red circles. The minimum spanning tree edges d-a, d-f, a-b, b-e, e-c, e-g are drawn thick red; remaining edges are thin black with integer weights.</t>
         </is>
       </c>
       <c r="D108" s="17" t="inlineStr">
@@ -3304,139 +3310,139 @@
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t>14.41</t>
+          <t>14.43</t>
         </is>
       </c>
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>Prim’s algorithm</t>
+          <t>Exercise diagram: a stylized neighborhood shown as six rectangular blocks in two rows of three.</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>Python code listing 'Loading the graph into NetworkX' that builds the prior 6-vertex weighted graph in NetworkX: it imports nx, creates an undirected Graph, adds nodes A,B,C,E,F,G, and feeds the 15 weighted edges via G.add_weighted_edges_from(edges).
-Five-vertex graph with cities A, B, C, D, E as black dots, fully connected with dollar-cost edge labels (AB=4, AE=5, AC=8, DC=7, plus higher cross-edges). Edges AB, AE, AC, DC are thick red, marking the MST built by Prim's algorithm starting at A.
-Same five-city phone-line graph (A, B, C, D, E) used to illustrate Prim's algorithm. Edges are labelled with dollar costs and the spanning tree edges AB, AE, AC, DC are drawn in thick red while the remaining inter-city edges are thin black.</t>
+          <t>Exercise diagram: a stylized neighborhood shown as six rectangular blocks in two rows of three. Black squares on the inside borders of each block mark houses; students draw edges along the streets the carrier walks to reach every house.</t>
         </is>
       </c>
       <c r="D109" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E109" s="17" t="inlineStr"/>
-      <c r="F109" s="17" t="inlineStr"/>
+          <t>CC BY-SA 3.0</t>
+        </is>
+      </c>
+      <c r="E109" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society: Graphexercise1</t>
+        </is>
+      </c>
+      <c r="F109" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society, "Graphexercise1", CC BY-SA 3.0</t>
+        </is>
+      </c>
       <c r="G109" s="17" t="inlineStr"/>
       <c r="H109" s="17" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
         <is>
-          <t>14.42</t>
+          <t>14.44</t>
         </is>
       </c>
       <c r="B110" s="17" t="inlineStr">
         <is>
-          <t>Boxed figure for Prim’s algorithm: 7-vertex graph with vertices a, b, c, d, e, f, g as red circles.</t>
+          <t>Exercise map of a fictional town: a teal river divides the area into several land masses, with...</t>
         </is>
       </c>
       <c r="C110" s="17" t="inlineStr">
         <is>
-          <t>Boxed figure for Prim's algorithm: 7-vertex graph with vertices a, b, c, d, e, f, g as red circles. The minimum spanning tree edges d-a, d-f, a-b, b-e, e-c, e-g are drawn thick red; remaining edges are thin black with integer weights.</t>
+          <t>Exercise map of a fictional town: a teal river divides the area into several land masses, with seven black bars marking bridges. Students convert the map to a graph to test for an Eulerian path crossing each bridge once.</t>
         </is>
       </c>
       <c r="D110" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E110" s="17" t="inlineStr"/>
-      <c r="F110" s="17" t="inlineStr"/>
+          <t>CC BY-SA 3.0</t>
+        </is>
+      </c>
+      <c r="E110" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society: Graphexercise2</t>
+        </is>
+      </c>
+      <c r="F110" s="17" t="inlineStr">
+        <is>
+          <t>David Lippman, Math in Society, "Graphexercise2", CC BY-SA 3.0</t>
+        </is>
+      </c>
       <c r="G110" s="17" t="inlineStr"/>
       <c r="H110" s="17" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
         <is>
-          <t>14.43</t>
+          <t>14.45</t>
         </is>
       </c>
       <c r="B111" s="17" t="inlineStr">
         <is>
-          <t>Exercise diagram: a stylized neighborhood shown as six rectangular blocks in two rows of three.</t>
+          <t>Five-vertex graph for the degree exercise.</t>
         </is>
       </c>
       <c r="C111" s="17" t="inlineStr">
         <is>
-          <t>Exercise diagram: a stylized neighborhood shown as six rectangular blocks in two rows of three. Black squares on the inside borders of each block mark houses; students draw edges along the streets the carrier walks to reach every house.</t>
+          <t>Seven-vertex weighted graph for the shortest-path exercise. Vertices A, B, C, D, E, F, G in a roughly diamond layout with integer edge weights (AB=1, AC=4, BD=3, CD=2, DE=2, DF=4, EG=7, FG=6, plus chords). Goal: find the shortest path from A to G.</t>
         </is>
       </c>
       <c r="D111" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 3.0</t>
-        </is>
-      </c>
-      <c r="E111" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society: Graphexercise1</t>
-        </is>
-      </c>
-      <c r="F111" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society, "Graphexercise1", CC BY-SA 3.0</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E111" s="17" t="inlineStr"/>
+      <c r="F111" s="17" t="inlineStr"/>
       <c r="G111" s="17" t="inlineStr"/>
       <c r="H111" s="17" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
         <is>
-          <t>14.44</t>
+          <t>14.46</t>
         </is>
       </c>
       <c r="B112" s="17" t="inlineStr">
         <is>
-          <t>Exercise map of a fictional town: a teal river divides the area into several land masses, with...</t>
+          <t>Another five-vertex graph for the degree exercise.</t>
         </is>
       </c>
       <c r="C112" s="17" t="inlineStr">
         <is>
-          <t>Exercise map of a fictional town: a teal river divides the area into several land masses, with seven black bars marking bridges. Students convert the map to a graph to test for an Eulerian path crossing each bridge once.</t>
+          <t>Airfare table giving one-way dollar fares between Seattle, Honolulu, London, Moscow, and Cairo (e.g. Seattle-Honolulu $159, Honolulu-London $830, London-Moscow $245, Moscow-Cairo $329). Used as input for building a weighted graph.</t>
         </is>
       </c>
       <c r="D112" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 3.0</t>
-        </is>
-      </c>
-      <c r="E112" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society: Graphexercise2</t>
-        </is>
-      </c>
-      <c r="F112" s="17" t="inlineStr">
-        <is>
-          <t>David Lippman, Math in Society, "Graphexercise2", CC BY-SA 3.0</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E112" s="17" t="inlineStr"/>
+      <c r="F112" s="17" t="inlineStr"/>
       <c r="G112" s="17" t="inlineStr"/>
       <c r="H112" s="17" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="16" t="inlineStr">
         <is>
-          <t>14.45</t>
+          <t>14.47</t>
         </is>
       </c>
       <c r="B113" s="17" t="inlineStr">
         <is>
-          <t>Seven-vertex weighted graph for the shortest-path exercise.</t>
+          <t>Three five-vertex graphs for the connectedness exercise.</t>
         </is>
       </c>
       <c r="C113" s="17" t="inlineStr">
         <is>
-          <t>Seven-vertex weighted graph for the shortest-path exercise. Vertices A, B, C, D, E, F, G in a roughly diamond layout with integer edge weights (AB=1, AC=4, BD=3, CD=2, DE=2, DF=4, EG=7, FG=6, plus chords). Goal: find the shortest path from A to G.</t>
+          <t>Small undirected graph with five black-dot vertices arranged in two rows, with four edges (square plus a diagonal extension). One of three example graphs presented side-by-side asking 'Which of these graphs are connected?'.
+Small undirected graph with five black-dot vertices; edges form one triangle on the right plus a separate vertical segment on the left, leaving the graph in two components. One of three connectivity examples.
+Small undirected graph with five black-dot vertices fully linked through a series of edges so all vertices belong to one component. The third option in the 'Which of these graphs are connected?' exercise.</t>
         </is>
       </c>
       <c r="D113" s="17" t="inlineStr">
@@ -3452,17 +3458,19 @@
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
         <is>
-          <t>14.46</t>
+          <t>14.48</t>
         </is>
       </c>
       <c r="B114" s="17" t="inlineStr">
         <is>
-          <t>Airfare table giving one-way dollar fares between Seattle, Honolulu, London, Moscow, and Cairo (e.g.</t>
+          <t>Three more graphs for the connectedness exercise.</t>
         </is>
       </c>
       <c r="C114" s="17" t="inlineStr">
         <is>
-          <t>Airfare table giving one-way dollar fares between Seattle, Honolulu, London, Moscow, and Cairo (e.g. Seattle-Honolulu $159, Honolulu-London $830, London-Moscow $245, Moscow-Cairo $329). Used as input for building a weighted graph.</t>
+          <t>Eight-vertex graph drawn on a 3-by-3 grid layout with three short horizontal segments stacked at top, middle, and bottom; the components are not all linked, illustrating a disconnected graph for the second connectivity question.
+Eight-vertex graph on a 3-by-3 grid layout where a central vertex (1.5,1) has high degree, connecting most of the graph; one corner pair remains separated. Used for the second 'Which of these graphs are connected?' question.
+Eight-vertex graph with edges forming a connected outer cycle plus several interior diagonals; the third option in the second connectivity exercise.</t>
         </is>
       </c>
       <c r="D114" s="17" t="inlineStr">
@@ -3478,19 +3486,17 @@
     <row r="115">
       <c r="A115" s="16" t="inlineStr">
         <is>
-          <t>14.47</t>
+          <t>14.49</t>
         </is>
       </c>
       <c r="B115" s="17" t="inlineStr">
         <is>
-          <t>Three five-vertex graphs for the connectedness exercise.</t>
+          <t>European rail network with travel times between cities.</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
         <is>
-          <t>Small undirected graph with five black-dot vertices arranged in two rows, with four edges (square plus a diagonal extension). One of three example graphs presented side-by-side asking 'Which of these graphs are connected?'.
-Small undirected graph with five black-dot vertices; edges form one triangle on the right plus a separate vertical segment on the left, leaving the graph in two components. One of three connectivity examples.
-Small undirected graph with five black-dot vertices fully linked through a series of edges so all vertices belong to one component. The third option in the 'Which of these graphs are connected?' exercise.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D115" s="17" t="inlineStr">
@@ -3506,19 +3512,17 @@
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
         <is>
-          <t>14.48</t>
+          <t>14.50</t>
         </is>
       </c>
       <c r="B116" s="17" t="inlineStr">
         <is>
-          <t>Three more graphs for the connectedness exercise.</t>
+          <t>Weighted graph on five labelled vertices A, B, C, D, E in a pentagonal layout, fully connected by...</t>
         </is>
       </c>
       <c r="C116" s="17" t="inlineStr">
         <is>
-          <t>Eight-vertex graph drawn on a 3-by-3 grid layout with three short horizontal segments stacked at top, middle, and bottom; the components are not all linked, illustrating a disconnected graph for the second connectivity question.
-Eight-vertex graph on a 3-by-3 grid layout where a central vertex (1.5,1) has high degree, connecting most of the graph; one corner pair remains separated. Used for the second 'Which of these graphs are connected?' question.
-Eight-vertex graph with edges forming a connected outer cycle plus several interior diagonals; the third option in the second connectivity exercise.</t>
+          <t>Weighted graph on five labelled vertices A, B, C, D, E in a pentagonal layout, fully connected by ten edges with dollar-cost labels (e.g. CD=$5.6, CA=$5.1, BC=$4.3, AE=$4.4, CE=$4.0); used to plan a minimum-cost sonet ring.</t>
         </is>
       </c>
       <c r="D116" s="17" t="inlineStr">
@@ -3534,17 +3538,17 @@
     <row r="117">
       <c r="A117" s="16" t="inlineStr">
         <is>
-          <t>14.49</t>
+          <t>14.51</t>
         </is>
       </c>
       <c r="B117" s="17" t="inlineStr">
         <is>
-          <t>European rail network with travel times between cities.</t>
+          <t>Virginia passenger rail network with travel times in minutes.</t>
         </is>
       </c>
       <c r="C117" s="17" t="inlineStr">
         <is>
-          <t>European rail network with travel times between cities.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D117" s="17" t="inlineStr">
@@ -3560,43 +3564,51 @@
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
         <is>
-          <t>14.50</t>
+          <t>15.1</t>
         </is>
       </c>
       <c r="B118" s="17" t="inlineStr">
         <is>
-          <t>Weighted graph on five labelled vertices A, B, C, D, E in a pentagonal layout, fully connected by...</t>
+          <t>Knapsack Problem: which items should we choose to take in the knapsack that maximizes the value while respecting the 15kg weight limit?</t>
         </is>
       </c>
       <c r="C118" s="17" t="inlineStr">
         <is>
-          <t>Weighted graph on five labelled vertices A, B, C, D, E in a pentagonal layout, fully connected by ten edges with dollar-cost labels (e.g. CD=$5.6, CA=$5.1, BC=$4.3, AE=$4.4, CE=$4.0); used to plan a minimum-cost sonet ring.</t>
+          <t>Illustration of the knapsack problem: a backpack with 15 kg capacity and a collection of boxes with different weights and dollar values, asking which boxes to select to maximize value.</t>
         </is>
       </c>
       <c r="D118" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E118" s="17" t="inlineStr"/>
-      <c r="F118" s="17" t="inlineStr"/>
+          <t>CC BY-SA 2.5</t>
+        </is>
+      </c>
+      <c r="E118" s="17" t="inlineStr">
+        <is>
+          <t>See page for author: Image of backpack and four blocks with different weight and value.</t>
+        </is>
+      </c>
+      <c r="F118" s="17" t="inlineStr">
+        <is>
+          <t>See page for author, "Image of backpack and four blocks with different weight and value.", CC BY-SA 2.5, https://en.wikipedia.org/wiki/Knapsack_problem</t>
+        </is>
+      </c>
       <c r="G118" s="17" t="inlineStr"/>
       <c r="H118" s="17" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="16" t="inlineStr">
         <is>
-          <t>14.51</t>
+          <t>15.2</t>
         </is>
       </c>
       <c r="B119" s="17" t="inlineStr">
         <is>
-          <t>Virginia cities road network with distances.</t>
+          <t>A network diagram for facility location: three potential distribution centers connected to stores.</t>
         </is>
       </c>
       <c r="C119" s="17" t="inlineStr">
         <is>
-          <t>Virginia cities road network with distances.</t>
+          <t>A network diagram for facility location showing three potential distribution centers with fixed costs and capacities, connected to four customer locations with demand values and shipping costs.</t>
         </is>
       </c>
       <c r="D119" s="17" t="inlineStr">
@@ -3612,51 +3624,43 @@
     <row r="120">
       <c r="A120" s="16" t="inlineStr">
         <is>
-          <t>15.1</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="B120" s="17" t="inlineStr">
         <is>
-          <t>Knapsack Problem: which items should we choose to take in the knapsack that maximizes the value while respecting the 15kg weight limit?</t>
+          <t>Layout of districts and possible locations of fire stations.</t>
         </is>
       </c>
       <c r="C120" s="17" t="inlineStr">
         <is>
-          <t>Illustration of the knapsack problem: a backpack with 15 kg capacity and a collection of boxes with different weights and dollar values, asking which boxes to select to maximize value.</t>
+          <t>Layout of districts showing numbered regions and possible locations for fire stations.</t>
         </is>
       </c>
       <c r="D120" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 2.5</t>
-        </is>
-      </c>
-      <c r="E120" s="17" t="inlineStr">
-        <is>
-          <t>See page for author: Image of backpack and four blocks with different weight and value.</t>
-        </is>
-      </c>
-      <c r="F120" s="17" t="inlineStr">
-        <is>
-          <t>See page for author, "Image of backpack and four blocks with different weight and value.", CC BY-SA 2.5, https://en.wikipedia.org/wiki/Knapsack_problem</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E120" s="17" t="inlineStr"/>
+      <c r="F120" s="17" t="inlineStr"/>
       <c r="G120" s="17" t="inlineStr"/>
       <c r="H120" s="17" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
         <is>
-          <t>15.2</t>
+          <t>15.4</t>
         </is>
       </c>
       <c r="B121" s="17" t="inlineStr">
         <is>
-          <t>A network diagram for facility location: three potential distribution centers connected to stores.</t>
+          <t>Set cover representation of fire station problem. For example, choosing district 16 to have a fire station covers districts 13, 15, and 16.</t>
         </is>
       </c>
       <c r="C121" s="17" t="inlineStr">
         <is>
-          <t>A network diagram for facility location showing three potential distribution centers with fixed costs and capacities, connected to four customer locations with demand values and shipping costs.</t>
+          <t>Set cover representation of fire station problem showing which districts are covered by each potential fire station location.</t>
         </is>
       </c>
       <c r="D121" s="17" t="inlineStr">
@@ -3672,17 +3676,17 @@
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="B122" s="17" t="inlineStr">
         <is>
-          <t>Layout of districts and possible locations of fire stations.</t>
+          <t>Graph representation of fire station problem. Every node is connected to a chosen node by an edge.</t>
         </is>
       </c>
       <c r="C122" s="17" t="inlineStr">
         <is>
-          <t>Layout of districts showing numbered regions and possible locations for fire stations.</t>
+          <t>Graph representation of fire station problem showing nodes connected to chosen fire station nodes by edges.</t>
         </is>
       </c>
       <c r="D122" s="17" t="inlineStr">
@@ -3698,43 +3702,51 @@
     <row r="123">
       <c r="A123" s="16" t="inlineStr">
         <is>
-          <t>15.4</t>
+          <t>15.6</t>
         </is>
       </c>
       <c r="B123" s="17" t="inlineStr">
         <is>
-          <t>Set cover representation of fire station problem. For example, choosing district 16 to have a fire station covers districts 13, 15, and 16.</t>
+          <t>A valid 3-coloring of the Petersen graph: no two adjacent vertices share a color.</t>
         </is>
       </c>
       <c r="C123" s="17" t="inlineStr">
         <is>
-          <t>Set cover representation of fire station problem showing which districts are covered by each potential fire station location.</t>
+          <t>Petersen graph with vertices colored using three colors (red, green, blue) demonstrating a valid 3-coloring where no adjacent vertices share the same color.</t>
         </is>
       </c>
       <c r="D123" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E123" s="17" t="inlineStr"/>
-      <c r="F123" s="17" t="inlineStr"/>
+          <t>Public domain</t>
+        </is>
+      </c>
+      <c r="E123" s="17" t="inlineStr">
+        <is>
+          <t>See page for author, via Wikimedia Commons: Petersen Graph 3-coloring</t>
+        </is>
+      </c>
+      <c r="F123" s="17" t="inlineStr">
+        <is>
+          <t>See page for author, via Wikimedia Commons, "Petersen Graph 3-coloring", Public domain, https://commons.wikimedia.org/wiki/File:Petersen_graph_3-coloring.svg</t>
+        </is>
+      </c>
       <c r="G123" s="17" t="inlineStr"/>
       <c r="H123" s="17" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="16" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>15.7</t>
         </is>
       </c>
       <c r="B124" s="17" t="inlineStr">
         <is>
-          <t>Graph representation of fire station problem. Every node is connected to a chosen node by an edge.</t>
+          <t>Simplified NYC Transportation Network with Directional Tolls</t>
         </is>
       </c>
       <c r="C124" s="17" t="inlineStr">
         <is>
-          <t>Graph representation of fire station problem showing nodes connected to chosen fire station nodes by edges.</t>
+          <t>Map of New York City's five boroughs showing a transportation network with red dashed toll roads and a green no-toll route connecting Staten Island, Brooklyn, and Queens.</t>
         </is>
       </c>
       <c r="D124" s="17" t="inlineStr">
@@ -3750,51 +3762,44 @@
     <row r="125">
       <c r="A125" s="16" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>15.8</t>
         </is>
       </c>
       <c r="B125" s="17" t="inlineStr">
         <is>
-          <t>A valid 3-coloring of the Petersen graph: no two adjacent vertices share a color.</t>
+          <t>An Example of the Strip Packing Problem</t>
         </is>
       </c>
       <c r="C125" s="17" t="inlineStr">
         <is>
-          <t>Petersen graph with vertices colored using three colors (red, green, blue) demonstrating a valid 3-coloring where no adjacent vertices share the same color.</t>
+          <t>Strip packing problem input showing four rectangles with their dimensions labeled, alongside an empty strip where they need to be packed.
+A strip packing diagram showing several gray rectangles of varying sizes packed within a vertical strip of width W, with a dotted horizontal line at height H indicating the current maximum height.</t>
         </is>
       </c>
       <c r="D125" s="17" t="inlineStr">
         <is>
-          <t>Public domain</t>
-        </is>
-      </c>
-      <c r="E125" s="17" t="inlineStr">
-        <is>
-          <t>See page for author, via Wikimedia Commons: Petersen Graph 3-coloring</t>
-        </is>
-      </c>
-      <c r="F125" s="17" t="inlineStr">
-        <is>
-          <t>See page for author, via Wikimedia Commons, "Petersen Graph 3-coloring", Public domain, https://commons.wikimedia.org/wiki/File:Petersen_graph_3-coloring.svg</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E125" s="17" t="inlineStr"/>
+      <c r="F125" s="17" t="inlineStr"/>
       <c r="G125" s="17" t="inlineStr"/>
       <c r="H125" s="17" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="16" t="inlineStr">
         <is>
-          <t>15.7</t>
+          <t>15.9</t>
         </is>
       </c>
       <c r="B126" s="17" t="inlineStr">
         <is>
-          <t>Simplified NYC Transportation Network with Directional Tolls</t>
+          <t>An optimal solution to the strip packing example.</t>
         </is>
       </c>
       <c r="C126" s="17" t="inlineStr">
         <is>
-          <t>Map of New York City's five boroughs showing a transportation network with red dashed toll roads and a green no-toll route connecting Staten Island, Brooklyn, and Queens.</t>
+          <t>A feasible strip packing solution showing rectangles packed into the strip with coordinate positions listed for each rectangle.</t>
         </is>
       </c>
       <c r="D126" s="17" t="inlineStr">
@@ -3810,18 +3815,17 @@
     <row r="127">
       <c r="A127" s="16" t="inlineStr">
         <is>
-          <t>15.8</t>
+          <t>15.10</t>
         </is>
       </c>
       <c r="B127" s="17" t="inlineStr">
         <is>
-          <t>An Example of the Strip Packing Problem</t>
+          <t>Piecewise linear function.</t>
         </is>
       </c>
       <c r="C127" s="17" t="inlineStr">
         <is>
-          <t>Strip packing problem input showing four rectangles with their dimensions labeled, alongside an empty strip where they need to be packed.
-A strip packing diagram showing several gray rectangles of varying sizes packed within a vertical strip of width W, with a dotted horizontal line at height H indicating the current maximum height.</t>
+          <t>Plot of a piecewise linear function composed of several line segments with breakpoints marked on the horizontal axis.</t>
         </is>
       </c>
       <c r="D127" s="17" t="inlineStr">
@@ -3837,17 +3841,17 @@
     <row r="128">
       <c r="A128" s="16" t="inlineStr">
         <is>
-          <t>15.9</t>
+          <t>15.11</t>
         </is>
       </c>
       <c r="B128" s="17" t="inlineStr">
         <is>
-          <t>An optimal solution to the strip packing example.</t>
+          <t>Job shop scheduling solution shown as a Gantt chart.</t>
         </is>
       </c>
       <c r="C128" s="17" t="inlineStr">
         <is>
-          <t>A feasible strip packing solution showing rectangles packed into the strip with coordinate positions listed for each rectangle.</t>
+          <t>Gantt chart showing a job shop scheduling solution with three machines processing five jobs over time. Colored horizontal bars represent job operations on each machine, demonstrating how jobs are sequenced to minimize makespan.</t>
         </is>
       </c>
       <c r="D128" s="17" t="inlineStr">
@@ -3863,17 +3867,17 @@
     <row r="129">
       <c r="A129" s="16" t="inlineStr">
         <is>
-          <t>15.10</t>
+          <t>15.12</t>
         </is>
       </c>
       <c r="B129" s="17" t="inlineStr">
         <is>
-          <t>Piecewise linear function.</t>
+          <t>Gantt chart of the Duplo job shop scheduling solution with three machines and four color-coded jobs.</t>
         </is>
       </c>
       <c r="C129" s="17" t="inlineStr">
         <is>
-          <t>Plot of a piecewise linear function composed of several line segments with breakpoints marked on the horizontal axis.</t>
+          <t>Gantt chart showing a Job Shop Scheduling Problem solution with three machines and four jobs represented by colored bars over a time horizon of 0 to 12 units.</t>
         </is>
       </c>
       <c r="D129" s="17" t="inlineStr">
@@ -3889,17 +3893,17 @@
     <row r="130">
       <c r="A130" s="16" t="inlineStr">
         <is>
-          <t>15.11</t>
+          <t>15.13</t>
         </is>
       </c>
       <c r="B130" s="17" t="inlineStr">
         <is>
-          <t>Job shop scheduling solution shown as a Gantt chart.</t>
+          <t>Photograph of Duplo building blocks arranged as a physical demonstration of the job shop schedule.</t>
         </is>
       </c>
       <c r="C130" s="17" t="inlineStr">
         <is>
-          <t>Gantt chart showing a job shop scheduling solution with three machines processing five jobs over time. Colored horizontal bars represent job operations on each machine, demonstrating how jobs are sequenced to minimize makespan.</t>
+          <t>Photograph of colorful Duplo building blocks arranged on a table, representing a physical demonstration of a job shop scheduling problem with blocks of different colors and sizes.</t>
         </is>
       </c>
       <c r="D130" s="17" t="inlineStr">
@@ -3915,17 +3919,17 @@
     <row r="131">
       <c r="A131" s="16" t="inlineStr">
         <is>
-          <t>15.12</t>
+          <t>A.1</t>
         </is>
       </c>
       <c r="B131" s="17" t="inlineStr">
         <is>
-          <t>Gantt chart of the Duplo job shop scheduling solution with three machines and four color-coded jobs.</t>
+          <t>Two-dimensional plot of the line y = 3x + 2 on x-y axes with a gridded background.</t>
         </is>
       </c>
       <c r="C131" s="17" t="inlineStr">
         <is>
-          <t>Gantt chart showing a Job Shop Scheduling Problem solution with three machines and four jobs represented by colored bars over a time horizon of 0 to 12 units.</t>
+          <t>Two-dimensional plot of the line y = 3x + 2 on x-y axes with a gridded background. Three labelled points (-1,-1), (0,2), and (1,5) lie on a blue line of slope 3 with y-intercept 2.</t>
         </is>
       </c>
       <c r="D131" s="17" t="inlineStr">
@@ -3941,17 +3945,17 @@
     <row r="132">
       <c r="A132" s="16" t="inlineStr">
         <is>
-          <t>15.13</t>
+          <t>A.2</t>
         </is>
       </c>
       <c r="B132" s="17" t="inlineStr">
         <is>
-          <t>Photograph of Duplo building blocks arranged as a physical demonstration of the job shop schedule.</t>
+          <t>Two-dimensional plot of the line 2x + y = 4 on gridded x-y axes.</t>
         </is>
       </c>
       <c r="C132" s="17" t="inlineStr">
         <is>
-          <t>Photograph of colorful Duplo building blocks arranged on a table, representing a physical demonstration of a job shop scheduling problem with blocks of different colors and sizes.</t>
+          <t>Two-dimensional plot of the line 2x + y = 4 on gridded x-y axes. A blue line passes through three labelled points (-1,6), (0,4), and (1,2), illustrating slope -2 and y-intercept 4.</t>
         </is>
       </c>
       <c r="D132" s="17" t="inlineStr">
@@ -3967,17 +3971,17 @@
     <row r="133">
       <c r="A133" s="16" t="inlineStr">
         <is>
-          <t>A.1</t>
+          <t>A.3</t>
         </is>
       </c>
       <c r="B133" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the line y = 3x + 2 on x-y axes with a gridded background.</t>
+          <t>A line through the intercepts (0,-2) and (3,0).</t>
         </is>
       </c>
       <c r="C133" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the line y = 3x + 2 on x-y axes with a gridded background. Three labelled points (-1,-1), (0,2), and (1,5) lie on a blue line of slope 3 with y-intercept 2.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D133" s="17" t="inlineStr">
@@ -3993,17 +3997,17 @@
     <row r="134">
       <c r="A134" s="16" t="inlineStr">
         <is>
-          <t>A.2</t>
+          <t>A.4</t>
         </is>
       </c>
       <c r="B134" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the line 2x + y = 4 on gridded x-y axes.</t>
+          <t>A line through the points (3,1), (5,2), and (7,3).</t>
         </is>
       </c>
       <c r="C134" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the line 2x + y = 4 on gridded x-y axes. A blue line passes through three labelled points (-1,6), (0,4), and (1,2), illustrating slope -2 and y-intercept 4.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D134" s="17" t="inlineStr">
@@ -4019,17 +4023,17 @@
     <row r="135">
       <c r="A135" s="16" t="inlineStr">
         <is>
-          <t>A.3</t>
+          <t>A.5</t>
         </is>
       </c>
       <c r="B135" s="17" t="inlineStr">
         <is>
-          <t>A line through the intercepts (0,-2) and (3,0).</t>
+          <t>Two-dimensional plot of the horizontal line y = 3 on gridded x-y axes.</t>
         </is>
       </c>
       <c r="C135" s="17" t="inlineStr">
         <is>
-          <t>A line through the intercepts (0,-2) and (3,0).</t>
+          <t>Two-dimensional plot of the horizontal line y = 3 on gridded x-y axes. The blue line is drawn parallel to the x-axis through the labelled y-intercept (0,3).</t>
         </is>
       </c>
       <c r="D135" s="17" t="inlineStr">
@@ -4045,17 +4049,17 @@
     <row r="136">
       <c r="A136" s="16" t="inlineStr">
         <is>
-          <t>A.4</t>
+          <t>A.6</t>
         </is>
       </c>
       <c r="B136" s="17" t="inlineStr">
         <is>
-          <t>A line through the points (3,1), (5,2), and (7,3).</t>
+          <t>Two-dimensional plot of the vertical line x = -2 on gridded x-y axes.</t>
         </is>
       </c>
       <c r="C136" s="17" t="inlineStr">
         <is>
-          <t>A line through the points (3,1), (5,2), and (7,3).</t>
+          <t>Two-dimensional plot of the vertical line x = -2 on gridded x-y axes. The blue line is drawn parallel to the y-axis through the labelled x-intercept (-2,0).</t>
         </is>
       </c>
       <c r="D136" s="17" t="inlineStr">
@@ -4071,17 +4075,17 @@
     <row r="137">
       <c r="A137" s="16" t="inlineStr">
         <is>
-          <t>A.5</t>
+          <t>A.7</t>
         </is>
       </c>
       <c r="B137" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the horizontal line y = 3 on gridded x-y axes.</t>
+          <t>Two-dimensional plot illustrating the slope of the line through (-2,3) and (4,-1) on x-y axes.</t>
         </is>
       </c>
       <c r="C137" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the horizontal line y = 3 on gridded x-y axes. The blue line is drawn parallel to the x-axis through the labelled y-intercept (0,3).</t>
+          <t>Two-dimensional plot illustrating the slope of the line through (-2,3) and (4,-1) on x-y axes. A blue line connects the two labelled points; green arrows mark a vertical drop of -4 and a horizontal run of 6, giving slope -2/3.</t>
         </is>
       </c>
       <c r="D137" s="17" t="inlineStr">
@@ -4097,17 +4101,17 @@
     <row r="138">
       <c r="A138" s="16" t="inlineStr">
         <is>
-          <t>A.6</t>
+          <t>A.8</t>
         </is>
       </c>
       <c r="B138" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the vertical line x = -2 on gridded x-y axes.</t>
+          <t>Two-dimensional plot of the line through (1,2) with slope -3/4 on gridded x-y axes.</t>
         </is>
       </c>
       <c r="C138" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the vertical line x = -2 on gridded x-y axes. The blue line is drawn parallel to the y-axis through the labelled x-intercept (-2,0).</t>
+          <t>Two-dimensional plot of the line through (1,2) with slope -3/4 on gridded x-y axes. A blue line passes through the labelled points (1,2) and (5,-1); green arrows indicate a vertical change of -3 and horizontal change of 4.</t>
         </is>
       </c>
       <c r="D138" s="17" t="inlineStr">
@@ -4123,17 +4127,17 @@
     <row r="139">
       <c r="A139" s="16" t="inlineStr">
         <is>
-          <t>A.7</t>
+          <t>A.9</t>
         </is>
       </c>
       <c r="B139" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot illustrating the slope of the line through (-2,3) and (4,-1) on x-y axes.</t>
+          <t>Two-dimensional plot of an equilibrium point.</t>
         </is>
       </c>
       <c r="C139" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot illustrating the slope of the line through (-2,3) and (4,-1) on x-y axes. A blue line connects the two labelled points; green arrows mark a vertical drop of -4 and a horizontal run of 6, giving slope -2/3.</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="D139" s="17" t="inlineStr">
@@ -4149,17 +4153,17 @@
     <row r="140">
       <c r="A140" s="16" t="inlineStr">
         <is>
-          <t>A.8</t>
+          <t>A.10</t>
         </is>
       </c>
       <c r="B140" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the line through (1,2) with slope -3/4 on gridded x-y axes.</t>
+          <t>Two-dimensional plot of a break-even point.</t>
         </is>
       </c>
       <c r="C140" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the line through (1,2) with slope -3/4 on gridded x-y axes. A blue line passes through the labelled points (1,2) and (5,-1); green arrows indicate a vertical change of -3 and horizontal change of 4.</t>
+          <t>Two-dimensional plot of a break-even point. The blue revenue line R = 5x and the red cost line C = 3x + 12 intersect at the labelled green point (6,30), with dashed lines marking Quantity = 6 and Cost/Revenue = 30.</t>
         </is>
       </c>
       <c r="D140" s="17" t="inlineStr">
@@ -4175,17 +4179,17 @@
     <row r="141">
       <c r="A141" s="16" t="inlineStr">
         <is>
-          <t>A.9</t>
+          <t>B.1</t>
         </is>
       </c>
       <c r="B141" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of an equilibrium point.</t>
+          <t>Three side-by-side 2D plots showing how two lines can intersect: ’One Solution’ (crossing at a...</t>
         </is>
       </c>
       <c r="C141" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of an equilibrium point. The blue upward supply line y = 3.5x - 14 and the red downward demand line y = -2.5x + 34 intersect at the labelled green point (8,14), with dashed lines dropping to Quantity = 8 and Price = 14.</t>
+          <t>Three side-by-side 2D plots showing how two lines can intersect: 'One Solution' (crossing at a single point), 'No Solutions' (parallel lines), and 'Infinitely Many Solutions' (a single line representing two coincident equations).</t>
         </is>
       </c>
       <c r="D141" s="17" t="inlineStr">
@@ -4201,17 +4205,17 @@
     <row r="142">
       <c r="A142" s="16" t="inlineStr">
         <is>
-          <t>A.10</t>
+          <t>B.2</t>
         </is>
       </c>
       <c r="B142" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of a break-even point.</t>
+          <t>Two-dimensional plot of the system x+y=3 and y-x=5: a green line and a blue line crossing at the...</t>
         </is>
       </c>
       <c r="C142" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of a break-even point. The blue revenue line R = 5x and the red cost line C = 3x + 12 intersect at the labelled green point (6,30), with dashed lines marking Quantity = 6 and Cost/Revenue = 30.</t>
+          <t>Two-dimensional plot of the system x+y=3 and y-x=5: a green line and a blue line crossing at the labelled point (x,y) = (-1,4), with helper lines dropped to the x- and y-axes to show the unique solution.</t>
         </is>
       </c>
       <c r="D142" s="17" t="inlineStr">
@@ -4227,17 +4231,17 @@
     <row r="143">
       <c r="A143" s="16" t="inlineStr">
         <is>
-          <t>B.1</t>
+          <t>B.3</t>
         </is>
       </c>
       <c r="B143" s="17" t="inlineStr">
         <is>
-          <t>Three side-by-side 2D plots showing how two lines can intersect: ’One Solution’ (crossing at a...</t>
+          <t>Two side-by-side two-dimensional plots showing three lines in the plane: on the left, three lines...</t>
         </is>
       </c>
       <c r="C143" s="17" t="inlineStr">
         <is>
-          <t>Three side-by-side 2D plots showing how two lines can intersect: 'One Solution' (crossing at a single point), 'No Solutions' (parallel lines), and 'Infinitely Many Solutions' (a single line representing two coincident equations).</t>
+          <t>Two side-by-side two-dimensional plots showing three lines in the plane: on the left, three lines that pairwise intersect but share no common point ('No Solution'); on the right, three lines all passing through a single marked point ('One Solution').</t>
         </is>
       </c>
       <c r="D143" s="17" t="inlineStr">
@@ -4253,64 +4257,80 @@
     <row r="144">
       <c r="A144" s="16" t="inlineStr">
         <is>
-          <t>B.2</t>
+          <t>B.4</t>
         </is>
       </c>
       <c r="B144" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the system x+y=3 and y-x=5: a green line and a blue line crossing at the...</t>
+          <t>Two planes intersecting in a line.</t>
         </is>
       </c>
       <c r="C144" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the system x+y=3 and y-x=5: a green line and a blue line crossing at the labelled point (x,y) = (-1,4), with helper lines dropped to the x- and y-axes to show the unique solution.</t>
+          <t>PICT</t>
         </is>
       </c>
       <c r="D144" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E144" s="17" t="inlineStr"/>
-      <c r="F144" s="17" t="inlineStr"/>
+          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
+        </is>
+      </c>
+      <c r="E144" s="17" t="inlineStr">
+        <is>
+          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
+        </is>
+      </c>
+      <c r="F144" s="17" t="inlineStr">
+        <is>
+          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
+        </is>
+      </c>
       <c r="G144" s="17" t="inlineStr"/>
       <c r="H144" s="17" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="16" t="inlineStr">
         <is>
-          <t>B.3</t>
+          <t>B.5</t>
         </is>
       </c>
       <c r="B145" s="17" t="inlineStr">
         <is>
-          <t>Two side-by-side two-dimensional plots showing three lines in the plane: on the left, three lines...</t>
+          <t>Three planes with no common point of intersection.</t>
         </is>
       </c>
       <c r="C145" s="17" t="inlineStr">
         <is>
-          <t>Two side-by-side two-dimensional plots showing three lines in the plane: on the left, three lines that pairwise intersect but share no common point ('No Solution'); on the right, three lines all passing through a single marked point ('One Solution').</t>
+          <t>PICT</t>
         </is>
       </c>
       <c r="D145" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E145" s="17" t="inlineStr"/>
-      <c r="F145" s="17" t="inlineStr"/>
+          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
+        </is>
+      </c>
+      <c r="E145" s="17" t="inlineStr">
+        <is>
+          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
+        </is>
+      </c>
+      <c r="F145" s="17" t="inlineStr">
+        <is>
+          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
+        </is>
+      </c>
       <c r="G145" s="17" t="inlineStr"/>
       <c r="H145" s="17" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="16" t="inlineStr">
         <is>
-          <t>B.4</t>
+          <t>B.6</t>
         </is>
       </c>
       <c r="B146" s="17" t="inlineStr">
         <is>
-          <t>Two planes intersecting in a line.</t>
+          <t>Three planes intersecting in a single point.</t>
         </is>
       </c>
       <c r="C146" s="17" t="inlineStr">
@@ -4339,12 +4359,12 @@
     <row r="147">
       <c r="A147" s="16" t="inlineStr">
         <is>
-          <t>B.5</t>
+          <t>B.7</t>
         </is>
       </c>
       <c r="B147" s="17" t="inlineStr">
         <is>
-          <t>Three planes with no common point of intersection.</t>
+          <t>A third plane through the line of intersection of two planes.</t>
         </is>
       </c>
       <c r="C147" s="17" t="inlineStr">
@@ -4373,85 +4393,69 @@
     <row r="148">
       <c r="A148" s="16" t="inlineStr">
         <is>
-          <t>B.6</t>
+          <t>D.1</t>
         </is>
       </c>
       <c r="B148" s="17" t="inlineStr">
         <is>
-          <t>Three planes intersecting in a single point.</t>
+          <t>Two-dimensional plot of the xy-plane showing two points P = (2,1) and Q = (-3,4) marked as red...</t>
         </is>
       </c>
       <c r="C148" s="17" t="inlineStr">
         <is>
-          <t>PICT</t>
+          <t>Two-dimensional plot of the xy-plane showing two points P = (2,1) and Q = (-3,4) marked as red dots, with light helper lines dropped to the axes to indicate each point's coordinates.</t>
         </is>
       </c>
       <c r="D148" s="17" t="inlineStr">
         <is>
-          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
-        </is>
-      </c>
-      <c r="E148" s="17" t="inlineStr">
-        <is>
-          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
-        </is>
-      </c>
-      <c r="F148" s="17" t="inlineStr">
-        <is>
-          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E148" s="17" t="inlineStr"/>
+      <c r="F148" s="17" t="inlineStr"/>
       <c r="G148" s="17" t="inlineStr"/>
       <c r="H148" s="17" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="16" t="inlineStr">
         <is>
-          <t>B.7</t>
+          <t>D.2</t>
         </is>
       </c>
       <c r="B149" s="17" t="inlineStr">
         <is>
-          <t>A third plane through the line of intersection of two planes.</t>
+          <t>Three-dimensional diagram of the position vector 0P: a thick blue arrow from the origin along the...</t>
         </is>
       </c>
       <c r="C149" s="17" t="inlineStr">
         <is>
-          <t>PICT</t>
+          <t>Three-dimensional diagram of the position vector 0P: a thick blue arrow from the origin along the x-, y-, z-axes to a red point P=(p_1,p_2,p_3), labelled with the column-vector form [p_1,p_2,p_3]^T.</t>
         </is>
       </c>
       <c r="D149" s="17" t="inlineStr">
         <is>
-          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
-        </is>
-      </c>
-      <c r="E149" s="17" t="inlineStr">
-        <is>
-          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
-        </is>
-      </c>
-      <c r="F149" s="17" t="inlineStr">
-        <is>
-          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E149" s="17" t="inlineStr"/>
+      <c r="F149" s="17" t="inlineStr"/>
       <c r="G149" s="17" t="inlineStr"/>
       <c r="H149" s="17" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="16" t="inlineStr">
         <is>
-          <t>D.1</t>
+          <t>D.3</t>
         </is>
       </c>
       <c r="B150" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the xy-plane showing two points P = (2,1) and Q = (-3,4) marked as red...</t>
+          <t>Three-dimensional diagram with two parallel blue arrows of equal length and direction: the position...</t>
         </is>
       </c>
       <c r="C150" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional plot of the xy-plane showing two points P = (2,1) and Q = (-3,4) marked as red dots, with light helper lines dropped to the axes to indicate each point's coordinates.</t>
+          <t>Three-dimensional diagram with two parallel blue arrows of equal length and direction: the position vector 0P from the origin and a translated copy AB from point A to point B, illustrating that translating a vector preserves its identity.</t>
         </is>
       </c>
       <c r="D150" s="17" t="inlineStr">
@@ -4467,17 +4471,17 @@
     <row r="151">
       <c r="A151" s="16" t="inlineStr">
         <is>
-          <t>D.2</t>
+          <t>D.4</t>
         </is>
       </c>
       <c r="B151" s="17" t="inlineStr">
         <is>
-          <t>Three-dimensional diagram of the position vector 0P: a thick blue arrow from the origin along the...</t>
+          <t>Two-dimensional vector diagram illustrating the tip-to-tail rule for vector addition: arrow u along...</t>
         </is>
       </c>
       <c r="C151" s="17" t="inlineStr">
         <is>
-          <t>Three-dimensional diagram of the position vector 0P: a thick blue arrow from the origin along the x-, y-, z-axes to a red point P=(p_1,p_2,p_3), labelled with the column-vector form [p_1,p_2,p_3]^T.</t>
+          <t>Two-dimensional vector diagram illustrating the tip-to-tail rule for vector addition: arrow u along the x-axis, arrow v starting at the tip of u and going to the upper right, and a third arrow from the tail of u to the tip of v labelled u+v.</t>
         </is>
       </c>
       <c r="D151" s="17" t="inlineStr">
@@ -4493,43 +4497,51 @@
     <row r="152">
       <c r="A152" s="16" t="inlineStr">
         <is>
-          <t>D.3</t>
+          <t>D.5</t>
         </is>
       </c>
       <c r="B152" s="17" t="inlineStr">
         <is>
-          <t>Three-dimensional diagram with two parallel blue arrows of equal length and direction: the position...</t>
+          <t>Vector addition in three dimensions: u + v as the diagonal of the parallelepiped.</t>
         </is>
       </c>
       <c r="C152" s="17" t="inlineStr">
         <is>
-          <t>Three-dimensional diagram with two parallel blue arrows of equal length and direction: the position vector 0P from the origin and a translated copy AB from point A to point B, illustrating that translating a vector preserves its identity.</t>
+          <t>PICT</t>
         </is>
       </c>
       <c r="D152" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E152" s="17" t="inlineStr"/>
-      <c r="F152" s="17" t="inlineStr"/>
+          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
+        </is>
+      </c>
+      <c r="E152" s="17" t="inlineStr">
+        <is>
+          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
+        </is>
+      </c>
+      <c r="F152" s="17" t="inlineStr">
+        <is>
+          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
+        </is>
+      </c>
       <c r="G152" s="17" t="inlineStr"/>
       <c r="H152" s="17" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="16" t="inlineStr">
         <is>
-          <t>D.4</t>
+          <t>D.6</t>
         </is>
       </c>
       <c r="B153" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram illustrating the tip-to-tail rule for vector addition: arrow u along...</t>
+          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as...</t>
         </is>
       </c>
       <c r="C153" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram illustrating the tip-to-tail rule for vector addition: arrow u along the x-axis, arrow v starting at the tip of u and going to the upper right, and a third arrow from the tail of u to the tip of v labelled u+v.</t>
+          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as separate arrows, presented as the setup for graphing the linear combinations u+2v and u-1/2 v.</t>
         </is>
       </c>
       <c r="D153" s="17" t="inlineStr">
@@ -4545,51 +4557,43 @@
     <row r="154">
       <c r="A154" s="16" t="inlineStr">
         <is>
-          <t>D.5</t>
+          <t>D.7</t>
         </is>
       </c>
       <c r="B154" s="17" t="inlineStr">
         <is>
-          <t>Vector addition in three dimensions: u + v as the diagonal of the parallelepiped.</t>
+          <t>Two-dimensional vector diagram of u+v drawn tip-to-tail: blue u from the origin to the upper right...</t>
         </is>
       </c>
       <c r="C154" s="17" t="inlineStr">
         <is>
-          <t>PICT</t>
+          <t>Two-dimensional vector diagram of u+v drawn tip-to-tail: blue u from the origin to the upper right, red v continuing from the tip of u, and the purple resultant u+v drawn from the tail of u to the tip of v.</t>
         </is>
       </c>
       <c r="D154" s="17" t="inlineStr">
         <is>
-          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
-        </is>
-      </c>
-      <c r="E154" s="17" t="inlineStr">
-        <is>
-          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
-        </is>
-      </c>
-      <c r="F154" s="17" t="inlineStr">
-        <is>
-          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E154" s="17" t="inlineStr"/>
+      <c r="F154" s="17" t="inlineStr"/>
       <c r="G154" s="17" t="inlineStr"/>
       <c r="H154" s="17" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="16" t="inlineStr">
         <is>
-          <t>D.6</t>
+          <t>D.8</t>
         </is>
       </c>
       <c r="B155" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as...</t>
+          <t>Two-dimensional vector diagram of u-v: blue u from the origin, red -v starting at the tip of u and...</t>
         </is>
       </c>
       <c r="C155" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as separate arrows, presented as the setup for graphing the linear combinations u+2v and u-1/2 v.</t>
+          <t>Two-dimensional vector diagram of u-v: blue u from the origin, red -v starting at the tip of u and pointing in the reverse direction of v, and a purple arrow from the origin to the tip of -v representing u-v=u+(-v).</t>
         </is>
       </c>
       <c r="D155" s="17" t="inlineStr">
@@ -4605,127 +4609,127 @@
     <row r="156">
       <c r="A156" s="16" t="inlineStr">
         <is>
-          <t>D.7</t>
+          <t>D.9</t>
         </is>
       </c>
       <c r="B156" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram of u+v drawn tip-to-tail: blue u from the origin to the upper right...</t>
+          <t>The distance between two points in the plane.</t>
         </is>
       </c>
       <c r="C156" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram of u+v drawn tip-to-tail: blue u from the origin to the upper right, red v continuing from the tip of u, and the purple resultant u+v drawn from the tail of u to the tip of v.</t>
+          <t>PICT</t>
         </is>
       </c>
       <c r="D156" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E156" s="17" t="inlineStr"/>
-      <c r="F156" s="17" t="inlineStr"/>
+          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
+        </is>
+      </c>
+      <c r="E156" s="17" t="inlineStr">
+        <is>
+          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
+        </is>
+      </c>
+      <c r="F156" s="17" t="inlineStr">
+        <is>
+          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
+        </is>
+      </c>
       <c r="G156" s="17" t="inlineStr"/>
       <c r="H156" s="17" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="16" t="inlineStr">
         <is>
-          <t>D.8</t>
+          <t>D.10</t>
         </is>
       </c>
       <c r="B157" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram of u-v: blue u from the origin, red -v starting at the tip of u and...</t>
+          <t>The distance between two points in three dimensions.</t>
         </is>
       </c>
       <c r="C157" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram of u-v: blue u from the origin, red -v starting at the tip of u and pointing in the reverse direction of v, and a purple arrow from the origin to the tip of -v representing u-v=u+(-v).</t>
+          <t>PICT</t>
         </is>
       </c>
       <c r="D157" s="17" t="inlineStr">
         <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E157" s="17" t="inlineStr"/>
-      <c r="F157" s="17" t="inlineStr"/>
+          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
+        </is>
+      </c>
+      <c r="E157" s="17" t="inlineStr">
+        <is>
+          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
+        </is>
+      </c>
+      <c r="F157" s="17" t="inlineStr">
+        <is>
+          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
+        </is>
+      </c>
       <c r="G157" s="17" t="inlineStr"/>
       <c r="H157" s="17" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="16" t="inlineStr">
         <is>
-          <t>D.9</t>
+          <t>D.11</t>
         </is>
       </c>
       <c r="B158" s="17" t="inlineStr">
         <is>
-          <t>The distance between two points in the plane.</t>
+          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as...</t>
         </is>
       </c>
       <c r="C158" s="17" t="inlineStr">
         <is>
-          <t>PICT</t>
+          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as separate arrows, presented as the setup for graphing the linear combinations u+2v and u-1/2 v.</t>
         </is>
       </c>
       <c r="D158" s="17" t="inlineStr">
         <is>
-          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
-        </is>
-      </c>
-      <c r="E158" s="17" t="inlineStr">
-        <is>
-          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
-        </is>
-      </c>
-      <c r="F158" s="17" t="inlineStr">
-        <is>
-          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E158" s="17" t="inlineStr"/>
+      <c r="F158" s="17" t="inlineStr"/>
       <c r="G158" s="17" t="inlineStr"/>
       <c r="H158" s="17" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="16" t="inlineStr">
         <is>
-          <t>D.10</t>
+          <t>D.12</t>
         </is>
       </c>
       <c r="B159" s="17" t="inlineStr">
         <is>
-          <t>The distance between two points in three dimensions.</t>
+          <t>Two-dimensional diagram showing scalar multiples of two vectors: blue vector u and its negative -u...</t>
         </is>
       </c>
       <c r="C159" s="17" t="inlineStr">
         <is>
-          <t>PICT</t>
+          <t>Two-dimensional diagram showing scalar multiples of two vectors: blue vector u and its negative -u (same length, opposite direction), plus red vector v together with 2v (twice as long, same direction) and -1/2 v (half-length, reversed).</t>
         </is>
       </c>
       <c r="D159" s="17" t="inlineStr">
         <is>
-          <t>CC BY 4.0 (adapted from A First Course in Linear Algebra, Kuttler/Lyryx)</t>
-        </is>
-      </c>
-      <c r="E159" s="17" t="inlineStr">
-        <is>
-          <t>Adapted from A First Course in Linear Algebra by Ken Kuttler (Lyryx Learning)</t>
-        </is>
-      </c>
-      <c r="F159" s="17" t="inlineStr">
-        <is>
-          <t>Ken Kuttler, A First Course in Linear Algebra, Lyryx Learning, CC BY 4.0, https://lyryx.com/first-course-linear-algebra/</t>
-        </is>
-      </c>
+          <t>CC BY-SA 4.0 (original figure created for this book)</t>
+        </is>
+      </c>
+      <c r="E159" s="17" t="inlineStr"/>
+      <c r="F159" s="17" t="inlineStr"/>
       <c r="G159" s="17" t="inlineStr"/>
       <c r="H159" s="17" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="16" t="inlineStr">
         <is>
-          <t>D.11</t>
+          <t>D.13</t>
         </is>
       </c>
       <c r="B160" s="17" t="inlineStr">
@@ -4751,17 +4755,17 @@
     <row r="161">
       <c r="A161" s="16" t="inlineStr">
         <is>
-          <t>D.12</t>
+          <t>D.14</t>
         </is>
       </c>
       <c r="B161" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional diagram showing scalar multiples of two vectors: blue vector u and its negative -u...</t>
+          <t>Two-dimensional vector diagram of the linear combination u + 2v: blue vector u from the origin, red...</t>
         </is>
       </c>
       <c r="C161" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional diagram showing scalar multiples of two vectors: blue vector u and its negative -u (same length, opposite direction), plus red vector v together with 2v (twice as long, same direction) and -1/2 v (half-length, reversed).</t>
+          <t>Two-dimensional vector diagram of the linear combination u + 2v: blue vector u from the origin, red vector 2v drawn tip-to-tail starting at u's head, and the purple resultant u+2v from the origin to the final tip.</t>
         </is>
       </c>
       <c r="D161" s="17" t="inlineStr">
@@ -4777,17 +4781,17 @@
     <row r="162">
       <c r="A162" s="16" t="inlineStr">
         <is>
-          <t>D.13</t>
+          <t>D.15</t>
         </is>
       </c>
       <c r="B162" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as...</t>
+          <t>Two-dimensional vector diagram of the linear combination u - 1/2 v: blue u from the origin, the...</t>
         </is>
       </c>
       <c r="C162" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional sketch of vectors u (blue, up and right) and v (red, down and right) drawn as separate arrows, presented as the setup for graphing the linear combinations u+2v and u-1/2 v.</t>
+          <t>Two-dimensional vector diagram of the linear combination u - 1/2 v: blue u from the origin, the short red vector -1/2 v placed tip-to-tail at u's head, and the purple resultant u - 1/2 v drawn from the origin to the final tip.</t>
         </is>
       </c>
       <c r="D162" s="17" t="inlineStr">
@@ -4803,17 +4807,17 @@
     <row r="163">
       <c r="A163" s="16" t="inlineStr">
         <is>
-          <t>D.14</t>
+          <t>D.16</t>
         </is>
       </c>
       <c r="B163" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram of the linear combination u + 2v: blue vector u from the origin, red...</t>
+          <t>Two-dimensional sketch of two vectors emanating from a common origin: a blue vector v pointing up...</t>
         </is>
       </c>
       <c r="C163" s="17" t="inlineStr">
         <is>
-          <t>Two-dimensional vector diagram of the linear combination u + 2v: blue vector u from the origin, red vector 2v drawn tip-to-tail starting at u's head, and the purple resultant u+2v from the origin to the final tip.</t>
+          <t>Two-dimensional sketch of two vectors emanating from a common origin: a blue vector v pointing up and to the right and a red vector u pointing down and to the right, with the included angle theta marked between them.</t>
         </is>
       </c>
       <c r="D163" s="17" t="inlineStr">
@@ -4826,58 +4830,6 @@
       <c r="G163" s="17" t="inlineStr"/>
       <c r="H163" s="17" t="inlineStr"/>
     </row>
-    <row r="164">
-      <c r="A164" s="16" t="inlineStr">
-        <is>
-          <t>D.15</t>
-        </is>
-      </c>
-      <c r="B164" s="17" t="inlineStr">
-        <is>
-          <t>Two-dimensional vector diagram of the linear combination u - 1/2 v: blue u from the origin, the...</t>
-        </is>
-      </c>
-      <c r="C164" s="17" t="inlineStr">
-        <is>
-          <t>Two-dimensional vector diagram of the linear combination u - 1/2 v: blue u from the origin, the short red vector -1/2 v placed tip-to-tail at u's head, and the purple resultant u - 1/2 v drawn from the origin to the final tip.</t>
-        </is>
-      </c>
-      <c r="D164" s="17" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E164" s="17" t="inlineStr"/>
-      <c r="F164" s="17" t="inlineStr"/>
-      <c r="G164" s="17" t="inlineStr"/>
-      <c r="H164" s="17" t="inlineStr"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="16" t="inlineStr">
-        <is>
-          <t>D.16</t>
-        </is>
-      </c>
-      <c r="B165" s="17" t="inlineStr">
-        <is>
-          <t>Two-dimensional sketch of two vectors emanating from a common origin: a blue vector v pointing up...</t>
-        </is>
-      </c>
-      <c r="C165" s="17" t="inlineStr">
-        <is>
-          <t>Two-dimensional sketch of two vectors emanating from a common origin: a blue vector v pointing up and to the right and a red vector u pointing down and to the right, with the included angle theta marked between them.</t>
-        </is>
-      </c>
-      <c r="D165" s="17" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0 (original figure created for this book)</t>
-        </is>
-      </c>
-      <c r="E165" s="17" t="inlineStr"/>
-      <c r="F165" s="17" t="inlineStr"/>
-      <c r="G165" s="17" t="inlineStr"/>
-      <c r="H165" s="17" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>